<commit_message>
Sonavox CICU2064021: break down each HS row by item
Description cell now lists every item type (client's Czech description
<- exact invoice description) with its qty, net/gross weight and EUR,
and each HS row is followed by collapsible sub-rows per invoice line
(part number). CELKEM sums only the HS rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDfNjvRhvE2vaNKifmBYbR
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sonavox_CICU2064021.xlsx
+++ b/output/HS_Code_Summary_Sonavox_CICU2064021.xlsx
@@ -21,7 +21,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="#,##0.000"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -40,8 +40,13 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -61,6 +66,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
     <fill>
@@ -95,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -104,10 +114,10 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -119,13 +129,31 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -137,11 +165,14 @@
     <xf numFmtId="4" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="2" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="2" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -514,16 +545,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -735,7 +766,8 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Subwoofer; Hotové reproduktory - ostatní</t>
+          <t>• Subwoofer  ← faktura: "Car Speaker" – 1 080 ks | NW 977,400 kg | GW 1 055,820 kg | 5 988,60 EUR
+• Hotové reproduktory - ostatní  ← faktura: "Car Speaker" – 1 860 ks | NW 1 086,000 kg | GW 1 195,000 kg | 16 278,34 EUR</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
@@ -750,412 +782,1653 @@
       <c r="H14" s="10" t="n">
         <v>22266.94</v>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I14" s="11" t="inlineStr">
         <is>
           <t>3 % (dle List1; ověřit TARIC)</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr"/>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="J14" s="11" t="inlineStr"/>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090') | List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
-      <c r="L14" s="6" t="inlineStr">
+      <c r="L14" s="11" t="inlineStr">
         <is>
           <t>IM-SW6515-VWCZ, IM-40138L-BMWCZ, IM-65220G-BYCZ, IM-SW6550-SKCZ, IM-65386-BYCZ, IM-65387-BYCZ, IM-40137L-BMWCZ</t>
         </is>
       </c>
-      <c r="M14" s="6" t="inlineStr">
+      <c r="M14" s="11" t="inlineStr">
         <is>
           <t>Hotové autoreproduktory bez skříně (8518 29). List1 klienta uvádí starší kód 8518 29 95 (3 %) – ověřit platný TARIC. Pokud by byly dodány ve skříni → 8518 21 00 (4,5 %).</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
+    <row r="15" outlineLevel="1">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C15" s="13" t="inlineStr">
+        <is>
+          <t>8518290090</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Subwoofer  ← faktura: "Car Speaker"</t>
+        </is>
+      </c>
+      <c r="E15" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="F15" s="15" t="n">
+        <v>313.2</v>
+      </c>
+      <c r="G15" s="15" t="n">
+        <v>350</v>
+      </c>
+      <c r="H15" s="16" t="n">
+        <v>2381.4</v>
+      </c>
+      <c r="I15" s="12" t="inlineStr"/>
+      <c r="J15" s="12" t="inlineStr"/>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>IM-SW6515-VWCZ</t>
+        </is>
+      </c>
+      <c r="M15" s="12" t="inlineStr"/>
+    </row>
+    <row r="16" outlineLevel="1">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C16" s="13" t="inlineStr">
+        <is>
+          <t>8518290090</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+        </is>
+      </c>
+      <c r="E16" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="F16" s="15" t="n">
+        <v>253.8</v>
+      </c>
+      <c r="G16" s="15" t="n">
+        <v>270</v>
+      </c>
+      <c r="H16" s="16" t="n">
+        <v>4594.21</v>
+      </c>
+      <c r="I16" s="12" t="inlineStr"/>
+      <c r="J16" s="12" t="inlineStr"/>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+        </is>
+      </c>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
+          <t>IM-40138L-BMWCZ</t>
+        </is>
+      </c>
+      <c r="M16" s="12" t="inlineStr"/>
+    </row>
+    <row r="17" outlineLevel="1">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C17" s="13" t="inlineStr">
+        <is>
+          <t>8518290090</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+        </is>
+      </c>
+      <c r="E17" s="14" t="n">
+        <v>360</v>
+      </c>
+      <c r="F17" s="15" t="n">
+        <v>270</v>
+      </c>
+      <c r="G17" s="15" t="n">
+        <v>308</v>
+      </c>
+      <c r="H17" s="16" t="n">
+        <v>3623.72</v>
+      </c>
+      <c r="I17" s="12" t="inlineStr"/>
+      <c r="J17" s="12" t="inlineStr"/>
+      <c r="K17" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>IM-65220G-BYCZ</t>
+        </is>
+      </c>
+      <c r="M17" s="12" t="inlineStr"/>
+    </row>
+    <row r="18" outlineLevel="1">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="inlineStr">
+        <is>
+          <t>8518290090</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>Subwoofer  ← faktura: "Car Speaker"</t>
+        </is>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="F18" s="15" t="n">
+        <v>664.2</v>
+      </c>
+      <c r="G18" s="15" t="n">
+        <v>705.8200000000001</v>
+      </c>
+      <c r="H18" s="16" t="n">
+        <v>3607.2</v>
+      </c>
+      <c r="I18" s="12" t="inlineStr"/>
+      <c r="J18" s="12" t="inlineStr"/>
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>IM-SW6550-SKCZ</t>
+        </is>
+      </c>
+      <c r="M18" s="12" t="inlineStr"/>
+    </row>
+    <row r="19" outlineLevel="1">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="inlineStr">
+        <is>
+          <t>8518290090</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+        </is>
+      </c>
+      <c r="E19" s="14" t="n">
+        <v>240</v>
+      </c>
+      <c r="F19" s="15" t="n">
+        <v>175.2</v>
+      </c>
+      <c r="G19" s="15" t="n">
+        <v>195</v>
+      </c>
+      <c r="H19" s="16" t="n">
+        <v>2058.46</v>
+      </c>
+      <c r="I19" s="12" t="inlineStr"/>
+      <c r="J19" s="12" t="inlineStr"/>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>IM-65386-BYCZ</t>
+        </is>
+      </c>
+      <c r="M19" s="12" t="inlineStr"/>
+    </row>
+    <row r="20" outlineLevel="1">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C20" s="13" t="inlineStr">
+        <is>
+          <t>8518290090</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+        </is>
+      </c>
+      <c r="E20" s="14" t="n">
+        <v>180</v>
+      </c>
+      <c r="F20" s="15" t="n">
+        <v>133.2</v>
+      </c>
+      <c r="G20" s="15" t="n">
+        <v>152</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>1802.86</v>
+      </c>
+      <c r="I20" s="12" t="inlineStr"/>
+      <c r="J20" s="12" t="inlineStr"/>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>IM-65387-BYCZ</t>
+        </is>
+      </c>
+      <c r="M20" s="12" t="inlineStr"/>
+    </row>
+    <row r="21" outlineLevel="1">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C21" s="13" t="inlineStr">
+        <is>
+          <t>8518290090</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+        </is>
+      </c>
+      <c r="E21" s="14" t="n">
+        <v>540</v>
+      </c>
+      <c r="F21" s="15" t="n">
+        <v>253.8</v>
+      </c>
+      <c r="G21" s="15" t="n">
+        <v>270</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>4199.09</v>
+      </c>
+      <c r="I21" s="12" t="inlineStr"/>
+      <c r="J21" s="12" t="inlineStr"/>
+      <c r="K21" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+        </is>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
+          <t>IM-40137L-BMWCZ</t>
+        </is>
+      </c>
+      <c r="M21" s="12" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
+      <c r="B22" s="6" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C22" s="7" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
-        </is>
-      </c>
-      <c r="E15" s="8" t="n">
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>• Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component" – 13 341 ks | NW 4 431,030 kg | GW 4 598,920 kg | 5 696,96 EUR</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="n">
         <v>13341</v>
       </c>
-      <c r="F15" s="9" t="n">
+      <c r="F22" s="9" t="n">
         <v>4431.03</v>
       </c>
-      <c r="G15" s="9" t="n">
+      <c r="G22" s="9" t="n">
         <v>4598.92</v>
       </c>
-      <c r="H15" s="10" t="n">
+      <c r="H22" s="10" t="n">
         <v>5696.96</v>
       </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="I22" s="11" t="inlineStr">
         <is>
           <t>0 %</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr"/>
-      <c r="K15" s="6" t="inlineStr">
+      <c r="J22" s="11" t="inlineStr"/>
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>List1 ř.2 (obecná položka)</t>
         </is>
       </c>
-      <c r="L15" s="6" t="inlineStr">
+      <c r="L22" s="11" t="inlineStr">
         <is>
           <t>212-8061-1-CZ, 212-65424-CZ, 212-65581-CZ</t>
         </is>
       </c>
-      <c r="M15" s="6" t="inlineStr">
+      <c r="M22" s="11" t="inlineStr">
         <is>
           <t>Díly 212-* = rodina magnetických obvodů (List1 ř.3: 212-65163-CZ neodym → 8518 9000 30). Pokud jsou neodymové, ověřit podpoložku 30.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+    <row r="23" outlineLevel="1">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component"</t>
+        </is>
+      </c>
+      <c r="E23" s="14" t="n">
+        <v>4608</v>
+      </c>
+      <c r="F23" s="15" t="n">
+        <v>2211.84</v>
+      </c>
+      <c r="G23" s="15" t="n">
+        <v>2312</v>
+      </c>
+      <c r="H23" s="16" t="n">
+        <v>3170.3</v>
+      </c>
+      <c r="I23" s="12" t="inlineStr"/>
+      <c r="J23" s="12" t="inlineStr"/>
+      <c r="K23" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.2 (obecná položka)</t>
+        </is>
+      </c>
+      <c r="L23" s="12" t="inlineStr">
+        <is>
+          <t>212-8061-1-CZ</t>
+        </is>
+      </c>
+      <c r="M23" s="12" t="inlineStr"/>
+    </row>
+    <row r="24" outlineLevel="1">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C24" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component"</t>
+        </is>
+      </c>
+      <c r="E24" s="14" t="n">
+        <v>7680</v>
+      </c>
+      <c r="F24" s="15" t="n">
+        <v>1766.4</v>
+      </c>
+      <c r="G24" s="15" t="n">
+        <v>1797.6</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <v>1831.68</v>
+      </c>
+      <c r="I24" s="12" t="inlineStr"/>
+      <c r="J24" s="12" t="inlineStr"/>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.2 (obecná položka)</t>
+        </is>
+      </c>
+      <c r="L24" s="12" t="inlineStr">
+        <is>
+          <t>212-65424-CZ</t>
+        </is>
+      </c>
+      <c r="M24" s="12" t="inlineStr"/>
+    </row>
+    <row r="25" outlineLevel="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-1</t>
+        </is>
+      </c>
+      <c r="C25" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component"</t>
+        </is>
+      </c>
+      <c r="E25" s="14" t="n">
+        <v>1053</v>
+      </c>
+      <c r="F25" s="15" t="n">
+        <v>452.79</v>
+      </c>
+      <c r="G25" s="15" t="n">
+        <v>489.32</v>
+      </c>
+      <c r="H25" s="16" t="n">
+        <v>694.98</v>
+      </c>
+      <c r="I25" s="12" t="inlineStr"/>
+      <c r="J25" s="12" t="inlineStr"/>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.2 (obecná položka)</t>
+        </is>
+      </c>
+      <c r="L25" s="12" t="inlineStr">
+        <is>
+          <t>212-65581-CZ</t>
+        </is>
+      </c>
+      <c r="M25" s="12" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="B26" s="6" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C16" s="7" t="inlineStr">
+      <c r="C26" s="7" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>ocelová deska; jádro magnetického obvodu; Středící membrána; Terminál; Membrána s vlnkou; Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
-        </is>
-      </c>
-      <c r="E16" s="8" t="n">
+      <c r="D26" s="6" t="inlineStr">
+        <is>
+          <t>• ocelová deska  ← faktura: "Front plate" – 3 000 ks | NW 222,000 kg | GW 225,430 kg | 309,90 EUR
+• jádro magnetického obvodu  ← faktura: "T-yoke" – 60 000 ks | NW 8 012,640 kg | GW 8 192,640 kg | 9 581,83 EUR
+• Středící membrána  ← faktura: "Spider" – 3 000 ks | NW 4,500 kg | GW 9,500 kg | 282,60 EUR
+• Terminál  ← faktura: "Terminal" – 300 000 ks | NW 150,000 kg | GW 160,000 kg | 3 810,00 EUR
+• Membrána s vlnkou  ← faktura: "Cone" – 34 000 ks | NW 68,000 kg | GW 130,000 kg | 12 437,20 EUR
+• Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker components" – 21 600 ks | NW 5 616,000 kg | GW 5 736,000 kg | 5 978,88 EUR</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="n">
         <v>421600</v>
       </c>
-      <c r="F16" s="9" t="n">
+      <c r="F26" s="9" t="n">
         <v>14073.14</v>
       </c>
-      <c r="G16" s="9" t="n">
+      <c r="G26" s="9" t="n">
         <v>14453.57</v>
       </c>
-      <c r="H16" s="10" t="n">
+      <c r="H26" s="10" t="n">
         <v>32400.41</v>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>0 %</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr"/>
-      <c r="K16" s="6" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr"/>
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>List2 ř.14 (+ dřívější JSD 85189000 00) | List2 ř.23 | List2 ř.7 | List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ) | List2 ř.8 / List1 ř.4 | List1 ř.2 (obecná položka)</t>
         </is>
       </c>
-      <c r="L16" s="6" t="inlineStr">
+      <c r="L26" s="11" t="inlineStr">
         <is>
           <t>040-65E4-C-CZ, 210-50D3-17.5TCR-CZ, 021-88E00-9-2-CZ, 181-40133-1SN-CZ, 181-40133-2SN-CZ, 140-35D14-44XP1-CZ, 015-S753215-Y30-KS-CZ, 210-66E2-24.5TCR-1-CZ</t>
         </is>
       </c>
-      <c r="M16" s="6" t="inlineStr">
+      <c r="M26" s="11" t="inlineStr">
         <is>
           <t>Front plate: List1/List2 uvádí 8518900090, ale dřívější JSD klienta (přední deska) = 85189000 00 – '90' byla čistá hmotnost. 015-S753215-Y30-KS-CZ: 'Y30' = třída feritu → pravděpodobně feritový magnet; dle Pozn. 2a k tř. XVI by mohl patřit pod 8505 19 – klient řadí magnety pod 8518900000 (List2 'MAGNET'). Ocelové díly (front plate, T-yoke) – viz melt and pour.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
+    <row r="27" outlineLevel="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C27" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>ocelová deska  ← faktura: "Front plate"</t>
+        </is>
+      </c>
+      <c r="E27" s="14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F27" s="15" t="n">
+        <v>222</v>
+      </c>
+      <c r="G27" s="15" t="n">
+        <v>225.43</v>
+      </c>
+      <c r="H27" s="16" t="n">
+        <v>309.9</v>
+      </c>
+      <c r="I27" s="12" t="inlineStr"/>
+      <c r="J27" s="12" t="inlineStr"/>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.14 (+ dřívější JSD 85189000 00)</t>
+        </is>
+      </c>
+      <c r="L27" s="12" t="inlineStr">
+        <is>
+          <t>040-65E4-C-CZ</t>
+        </is>
+      </c>
+      <c r="M27" s="12" t="inlineStr"/>
+    </row>
+    <row r="28" outlineLevel="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>jádro magnetického obvodu  ← faktura: "T-yoke"</t>
+        </is>
+      </c>
+      <c r="E28" s="14" t="n">
+        <v>17160</v>
+      </c>
+      <c r="F28" s="15" t="n">
+        <v>1115.4</v>
+      </c>
+      <c r="G28" s="15" t="n">
+        <v>1155.4</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <v>1395.11</v>
+      </c>
+      <c r="I28" s="12" t="inlineStr"/>
+      <c r="J28" s="12" t="inlineStr"/>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.23</t>
+        </is>
+      </c>
+      <c r="L28" s="12" t="inlineStr">
+        <is>
+          <t>210-50D3-17.5TCR-CZ</t>
+        </is>
+      </c>
+      <c r="M28" s="12" t="inlineStr"/>
+    </row>
+    <row r="29" outlineLevel="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>Středící membrána  ← faktura: "Spider"</t>
+        </is>
+      </c>
+      <c r="E29" s="14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F29" s="15" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G29" s="15" t="n">
+        <v>9.5</v>
+      </c>
+      <c r="H29" s="16" t="n">
+        <v>282.6</v>
+      </c>
+      <c r="I29" s="12" t="inlineStr"/>
+      <c r="J29" s="12" t="inlineStr"/>
+      <c r="K29" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.7</t>
+        </is>
+      </c>
+      <c r="L29" s="12" t="inlineStr">
+        <is>
+          <t>021-88E00-9-2-CZ</t>
+        </is>
+      </c>
+      <c r="M29" s="12" t="inlineStr"/>
+    </row>
+    <row r="30" outlineLevel="1">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C30" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>Terminál  ← faktura: "Terminal"</t>
+        </is>
+      </c>
+      <c r="E30" s="14" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F30" s="15" t="n">
+        <v>75</v>
+      </c>
+      <c r="G30" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="H30" s="16" t="n">
+        <v>1905</v>
+      </c>
+      <c r="I30" s="12" t="inlineStr"/>
+      <c r="J30" s="12" t="inlineStr"/>
+      <c r="K30" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ)</t>
+        </is>
+      </c>
+      <c r="L30" s="12" t="inlineStr">
+        <is>
+          <t>181-40133-1SN-CZ</t>
+        </is>
+      </c>
+      <c r="M30" s="12" t="inlineStr"/>
+    </row>
+    <row r="31" outlineLevel="1">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C31" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Terminál  ← faktura: "Terminal"</t>
+        </is>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>150000</v>
+      </c>
+      <c r="F31" s="15" t="n">
+        <v>75</v>
+      </c>
+      <c r="G31" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="H31" s="16" t="n">
+        <v>1905</v>
+      </c>
+      <c r="I31" s="12" t="inlineStr"/>
+      <c r="J31" s="12" t="inlineStr"/>
+      <c r="K31" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ)</t>
+        </is>
+      </c>
+      <c r="L31" s="12" t="inlineStr">
+        <is>
+          <t>181-40133-2SN-CZ</t>
+        </is>
+      </c>
+      <c r="M31" s="12" t="inlineStr"/>
+    </row>
+    <row r="32" outlineLevel="1">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C32" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Membrána s vlnkou  ← faktura: "Cone"</t>
+        </is>
+      </c>
+      <c r="E32" s="14" t="n">
+        <v>34000</v>
+      </c>
+      <c r="F32" s="15" t="n">
+        <v>68</v>
+      </c>
+      <c r="G32" s="15" t="n">
+        <v>130</v>
+      </c>
+      <c r="H32" s="16" t="n">
+        <v>12437.2</v>
+      </c>
+      <c r="I32" s="12" t="inlineStr"/>
+      <c r="J32" s="12" t="inlineStr"/>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.8 / List1 ř.4</t>
+        </is>
+      </c>
+      <c r="L32" s="12" t="inlineStr">
+        <is>
+          <t>140-35D14-44XP1-CZ</t>
+        </is>
+      </c>
+      <c r="M32" s="12" t="inlineStr"/>
+    </row>
+    <row r="33" outlineLevel="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C33" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker components"</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="n">
+        <v>21600</v>
+      </c>
+      <c r="F33" s="15" t="n">
+        <v>5616</v>
+      </c>
+      <c r="G33" s="15" t="n">
+        <v>5736</v>
+      </c>
+      <c r="H33" s="16" t="n">
+        <v>5978.88</v>
+      </c>
+      <c r="I33" s="12" t="inlineStr"/>
+      <c r="J33" s="12" t="inlineStr"/>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>List1 ř.2 (obecná položka)</t>
+        </is>
+      </c>
+      <c r="L33" s="12" t="inlineStr">
+        <is>
+          <t>015-S753215-Y30-KS-CZ</t>
+        </is>
+      </c>
+      <c r="M33" s="12" t="inlineStr"/>
+    </row>
+    <row r="34" outlineLevel="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C34" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>jádro magnetického obvodu  ← faktura: "T-yoke"</t>
+        </is>
+      </c>
+      <c r="E34" s="14" t="n">
+        <v>42840</v>
+      </c>
+      <c r="F34" s="15" t="n">
+        <v>6897.24</v>
+      </c>
+      <c r="G34" s="15" t="n">
+        <v>7037.24</v>
+      </c>
+      <c r="H34" s="16" t="n">
+        <v>8186.72</v>
+      </c>
+      <c r="I34" s="12" t="inlineStr"/>
+      <c r="J34" s="12" t="inlineStr"/>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.23</t>
+        </is>
+      </c>
+      <c r="L34" s="12" t="inlineStr">
+        <is>
+          <t>210-66E2-24.5TCR-1-CZ</t>
+        </is>
+      </c>
+      <c r="M34" s="12" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="B35" s="6" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>3926909790</t>
         </is>
       </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>plastové těsnění</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="n">
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>• plastové těsnění  ← faktura: "Gasket" – 6 000 ks | NW 45,000 kg | GW 55,000 kg | 270,00 EUR</t>
+        </is>
+      </c>
+      <c r="E35" s="8" t="n">
         <v>6000</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F35" s="9" t="n">
         <v>45</v>
       </c>
-      <c r="G17" s="9" t="n">
+      <c r="G35" s="9" t="n">
         <v>55</v>
       </c>
-      <c r="H17" s="10" t="n">
+      <c r="H35" s="10" t="n">
         <v>270</v>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I35" s="11" t="inlineStr">
         <is>
           <t>6,5 %</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr">
+      <c r="J35" s="11" t="inlineStr"/>
+      <c r="K35" s="11" t="inlineStr">
         <is>
           <t>List2 ř.50 (39269097); díly 142-*, ne 143-* (gumové)</t>
         </is>
       </c>
-      <c r="L17" s="6" t="inlineStr">
+      <c r="L35" s="11" t="inlineStr">
         <is>
           <t>142-530H10-10H-CZ, 142-65580-3A-CZ</t>
         </is>
       </c>
-      <c r="M17" s="6" t="inlineStr">
+      <c r="M35" s="11" t="inlineStr">
         <is>
           <t>Materiál těsnění nepotvrzen. Plast → 3926 90 97 (6,5 %); pokud pryž → 4016 (List1 'Těsnění 40161000'); pěna → 3921. Ověřit.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+    <row r="36" outlineLevel="1">
+      <c r="A36" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C36" s="13" t="inlineStr">
+        <is>
+          <t>3926909790</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>plastové těsnění  ← faktura: "Gasket"</t>
+        </is>
+      </c>
+      <c r="E36" s="14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F36" s="15" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G36" s="15" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H36" s="16" t="n">
+        <v>126</v>
+      </c>
+      <c r="I36" s="12" t="inlineStr"/>
+      <c r="J36" s="12" t="inlineStr"/>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.50 (39269097); díly 142-*, ne 143-* (gumové)</t>
+        </is>
+      </c>
+      <c r="L36" s="12" t="inlineStr">
+        <is>
+          <t>142-530H10-10H-CZ</t>
+        </is>
+      </c>
+      <c r="M36" s="12" t="inlineStr"/>
+    </row>
+    <row r="37" outlineLevel="1">
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C37" s="13" t="inlineStr">
+        <is>
+          <t>3926909790</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>plastové těsnění  ← faktura: "Gasket"</t>
+        </is>
+      </c>
+      <c r="E37" s="14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F37" s="15" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G37" s="15" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H37" s="16" t="n">
+        <v>144</v>
+      </c>
+      <c r="I37" s="12" t="inlineStr"/>
+      <c r="J37" s="12" t="inlineStr"/>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.50 (39269097); díly 142-*, ne 143-* (gumové)</t>
+        </is>
+      </c>
+      <c r="L37" s="12" t="inlineStr">
+        <is>
+          <t>142-65580-3A-CZ</t>
+        </is>
+      </c>
+      <c r="M37" s="12" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="18" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B38" s="18" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C18" s="13" t="inlineStr">
+      <c r="C38" s="19" t="inlineStr">
         <is>
           <t>7318169290</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>Nut</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="n">
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>• Nut  ← faktura: "Nut" – 100 000 ks | NW 166,500 kg | GW 172,500 kg | 7 000,00 EUR</t>
+        </is>
+      </c>
+      <c r="E38" s="20" t="n">
         <v>100000</v>
       </c>
-      <c r="F18" s="15" t="n">
+      <c r="F38" s="21" t="n">
         <v>166.5</v>
       </c>
-      <c r="G18" s="15" t="n">
+      <c r="G38" s="21" t="n">
         <v>172.5</v>
       </c>
-      <c r="H18" s="16" t="n">
+      <c r="H38" s="22" t="n">
         <v>7000</v>
       </c>
-      <c r="I18" s="12" t="inlineStr">
+      <c r="I38" s="23" t="inlineStr">
         <is>
           <t>3,7 %</t>
         </is>
       </c>
-      <c r="J18" s="12" t="inlineStr">
+      <c r="J38" s="23" t="inlineStr">
         <is>
           <t>CBAM, MELT&amp;POUR</t>
         </is>
       </c>
-      <c r="K18" s="12" t="inlineStr">
+      <c r="K38" s="23" t="inlineStr">
         <is>
           <t>List2 ř.202 ('tohle řadíme pod 7318169290') – bez CZ popisu</t>
         </is>
       </c>
-      <c r="L18" s="12" t="inlineStr">
+      <c r="L38" s="23" t="inlineStr">
         <is>
           <t>029-2513-AL-CZ</t>
         </is>
       </c>
-      <c r="M18" s="12" t="inlineStr">
+      <c r="M38" s="23" t="inlineStr">
         <is>
           <t>CBAM zboží (ocelové matice, kap. 73). Příjemce v registru: Y137 (do 50 t ročně). Díl 029-2513-AL-CZ – přípona 'AL' může znamenat HLINÍK → pak 7616 10 00 (také CBAM). Antidumping na spojovací prvky z CN (nař. 2022/191) se týká šroubů/vrutů, NE matic 7318 16 → AD neočekáváno (ověřit). Melt and pour: hutní atest CHYBÍ.</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
+    <row r="39" outlineLevel="1">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904</t>
+        </is>
+      </c>
+      <c r="C39" s="13" t="inlineStr">
+        <is>
+          <t>7318169290</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>Nut  ← faktura: "Nut"</t>
+        </is>
+      </c>
+      <c r="E39" s="14" t="n">
+        <v>100000</v>
+      </c>
+      <c r="F39" s="15" t="n">
+        <v>166.5</v>
+      </c>
+      <c r="G39" s="15" t="n">
+        <v>172.5</v>
+      </c>
+      <c r="H39" s="16" t="n">
+        <v>7000</v>
+      </c>
+      <c r="I39" s="12" t="inlineStr"/>
+      <c r="J39" s="12" t="inlineStr"/>
+      <c r="K39" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.202 ('tohle řadíme pod 7318169290') – bez CZ popisu</t>
+        </is>
+      </c>
+      <c r="L39" s="12" t="inlineStr">
+        <is>
+          <t>029-2513-AL-CZ</t>
+        </is>
+      </c>
+      <c r="M39" s="12" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B19" s="6" t="inlineStr">
+      <c r="B40" s="6" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C40" s="7" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>Membrána s vlnkou; Kopulka= krycí vložka</t>
-        </is>
-      </c>
-      <c r="E19" s="8" t="n">
+      <c r="D40" s="6" t="inlineStr">
+        <is>
+          <t>• Membrána s vlnkou  ← faktura: "Cone" – 58 680 ks | NW 964,310 kg | GW 1 324,030 kg | 22 202,70 EUR
+• Kopulka= krycí vložka  ← faktura: "Dust cap" – 52 000 ks | NW 12,600 kg | GW 17,100 kg | 8 034,00 EUR</t>
+        </is>
+      </c>
+      <c r="E40" s="8" t="n">
         <v>110680</v>
       </c>
-      <c r="F19" s="9" t="n">
+      <c r="F40" s="9" t="n">
         <v>976.91</v>
       </c>
-      <c r="G19" s="9" t="n">
+      <c r="G40" s="9" t="n">
         <v>1341.13</v>
       </c>
-      <c r="H19" s="10" t="n">
+      <c r="H40" s="10" t="n">
         <v>30236.7</v>
       </c>
-      <c r="I19" s="6" t="inlineStr">
+      <c r="I40" s="11" t="inlineStr">
         <is>
           <t>0 %</t>
         </is>
       </c>
-      <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr">
+      <c r="J40" s="11" t="inlineStr"/>
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4 | List2 ř.9 (uvedeno 8518 9000 99)</t>
         </is>
       </c>
-      <c r="L19" s="6" t="inlineStr">
+      <c r="L40" s="11" t="inlineStr">
         <is>
           <t>140-65D24-179X-CZ, 140-80I27-42X-CZ, 160-B29-H-CZ, 140-65E22-203X-CZ, 140-40E17-72XC-CZ</t>
         </is>
       </c>
-      <c r="M19" s="6" t="inlineStr">
+      <c r="M40" s="11" t="inlineStr">
         <is>
           <t>Dust cap: List2 uvádí 8518 9000 99 – sloučeno pod 8518900000 (ostatní díly 8518 90 00), ověřit.</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+    <row r="41" outlineLevel="1">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-2</t>
+        </is>
+      </c>
+      <c r="C41" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>Membrána s vlnkou  ← faktura: "Cone"</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="n">
+        <v>17280</v>
+      </c>
+      <c r="F41" s="15" t="n">
+        <v>240</v>
+      </c>
+      <c r="G41" s="15" t="n">
+        <v>373.33</v>
+      </c>
+      <c r="H41" s="16" t="n">
+        <v>4397.76</v>
+      </c>
+      <c r="I41" s="12" t="inlineStr"/>
+      <c r="J41" s="12" t="inlineStr"/>
+      <c r="K41" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.8 / List1 ř.4</t>
+        </is>
+      </c>
+      <c r="L41" s="12" t="inlineStr">
+        <is>
+          <t>140-65D24-179X-CZ</t>
+        </is>
+      </c>
+      <c r="M41" s="12" t="inlineStr"/>
+    </row>
+    <row r="42" outlineLevel="1">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-2</t>
+        </is>
+      </c>
+      <c r="C42" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Membrána s vlnkou  ← faktura: "Cone"</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="n">
+        <v>24000</v>
+      </c>
+      <c r="F42" s="15" t="n">
+        <v>612</v>
+      </c>
+      <c r="G42" s="15" t="n">
+        <v>810</v>
+      </c>
+      <c r="H42" s="16" t="n">
+        <v>12026.4</v>
+      </c>
+      <c r="I42" s="12" t="inlineStr"/>
+      <c r="J42" s="12" t="inlineStr"/>
+      <c r="K42" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.8 / List1 ř.4</t>
+        </is>
+      </c>
+      <c r="L42" s="12" t="inlineStr">
+        <is>
+          <t>140-80I27-42X-CZ</t>
+        </is>
+      </c>
+      <c r="M42" s="12" t="inlineStr"/>
+    </row>
+    <row r="43" outlineLevel="1">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-2</t>
+        </is>
+      </c>
+      <c r="C43" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>Kopulka= krycí vložka  ← faktura: "Dust cap"</t>
+        </is>
+      </c>
+      <c r="E43" s="14" t="n">
+        <v>52000</v>
+      </c>
+      <c r="F43" s="15" t="n">
+        <v>12.6</v>
+      </c>
+      <c r="G43" s="15" t="n">
+        <v>17.1</v>
+      </c>
+      <c r="H43" s="16" t="n">
+        <v>8034</v>
+      </c>
+      <c r="I43" s="12" t="inlineStr"/>
+      <c r="J43" s="12" t="inlineStr"/>
+      <c r="K43" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.9 (uvedeno 8518 9000 99)</t>
+        </is>
+      </c>
+      <c r="L43" s="12" t="inlineStr">
+        <is>
+          <t>160-B29-H-CZ</t>
+        </is>
+      </c>
+      <c r="M43" s="12" t="inlineStr"/>
+    </row>
+    <row r="44" outlineLevel="1">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-2</t>
+        </is>
+      </c>
+      <c r="C44" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>Membrána s vlnkou  ← faktura: "Cone"</t>
+        </is>
+      </c>
+      <c r="E44" s="14" t="n">
+        <v>3000</v>
+      </c>
+      <c r="F44" s="15" t="n">
+        <v>25.91</v>
+      </c>
+      <c r="G44" s="15" t="n">
+        <v>39.36</v>
+      </c>
+      <c r="H44" s="16" t="n">
+        <v>895.5</v>
+      </c>
+      <c r="I44" s="12" t="inlineStr"/>
+      <c r="J44" s="12" t="inlineStr"/>
+      <c r="K44" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.8 / List1 ř.4</t>
+        </is>
+      </c>
+      <c r="L44" s="12" t="inlineStr">
+        <is>
+          <t>140-65E22-203X-CZ</t>
+        </is>
+      </c>
+      <c r="M44" s="12" t="inlineStr"/>
+    </row>
+    <row r="45" outlineLevel="1">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ↳ položka faktury</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="inlineStr">
+        <is>
+          <t>CZ20260904-2</t>
+        </is>
+      </c>
+      <c r="C45" s="13" t="inlineStr">
+        <is>
+          <t>8518900000</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>Membrána s vlnkou  ← faktura: "Cone"</t>
+        </is>
+      </c>
+      <c r="E45" s="14" t="n">
+        <v>14400</v>
+      </c>
+      <c r="F45" s="15" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="G45" s="15" t="n">
+        <v>101.34</v>
+      </c>
+      <c r="H45" s="16" t="n">
+        <v>4883.04</v>
+      </c>
+      <c r="I45" s="12" t="inlineStr"/>
+      <c r="J45" s="12" t="inlineStr"/>
+      <c r="K45" s="12" t="inlineStr">
+        <is>
+          <t>List2 ř.8 / List1 ř.4</t>
+        </is>
+      </c>
+      <c r="L45" s="12" t="inlineStr">
+        <is>
+          <t>140-40E17-72XC-CZ</t>
+        </is>
+      </c>
+      <c r="M45" s="12" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="24" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B20" s="18" t="n"/>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
-      <c r="E20" s="19">
-        <f>SUM(E14:E19)</f>
+      <c r="B46" s="25" t="n"/>
+      <c r="C46" s="25" t="n"/>
+      <c r="D46" s="25" t="n"/>
+      <c r="E46" s="26">
+        <f>E14+E22+E26+E35+E38+E40</f>
         <v/>
       </c>
-      <c r="F20" s="20">
-        <f>SUM(F14:F19)</f>
+      <c r="F46" s="27">
+        <f>F14+F22+F26+F35+F38+F40</f>
         <v/>
       </c>
-      <c r="G20" s="20">
-        <f>SUM(G14:G19)</f>
+      <c r="G46" s="27">
+        <f>G14+G22+G26+G35+G38+G40</f>
         <v/>
       </c>
-      <c r="H20" s="21">
-        <f>SUM(H14:H19)</f>
+      <c r="H46" s="28">
+        <f>H14+H22+H26+H35+H38+H40</f>
         <v/>
       </c>
-      <c r="I20" s="18" t="n"/>
-      <c r="J20" s="18" t="n"/>
-      <c r="K20" s="18" t="n"/>
-      <c r="L20" s="18" t="n"/>
-      <c r="M20" s="18" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
+      <c r="I46" s="25" t="n"/>
+      <c r="J46" s="25" t="n"/>
+      <c r="K46" s="25" t="n"/>
+      <c r="L46" s="25" t="n"/>
+      <c r="M46" s="25" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>Kontrola GW</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B48" t="inlineStr">
         <is>
           <t>Součet hrubých hmotností 22 871,94 kg = FCR TECGO26090103 i CIM 38272351 (22 871,94 kg) ✓</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>Hodnota (Total)</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>CZ20260904-1: 'Total Amount' 27 963,90. CZ20260904 a CZ20260904-2: pole 'Total Amount' je PRÁZDNÉ → použit 'Sub Total' (39 670,41 / 30 236,70; Duty/Freight/Insurance prázdné, sleva žádná)</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>Celní hodnota</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B50" t="inlineStr">
         <is>
           <t>Dodací podmínka FOB → k hodnotě připočíst dopravu po hranici EU (Malaszewicze) dle metodiky klienta</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Rozpis</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Pod každým HS řádkem (tučně) jsou šedé řádky ↳ = jednotlivé položky faktury: popis klienta (CZ) ← přesný popis z faktury, part number, ks, hmotnosti, EUR. CELKEM sčítá jen HS řádky. Řádky lze sbalit tlačítkem − vlevo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>🟡 žlutá</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B52" t="inlineStr">
         <is>
           <t>CBAM zboží – uvést Y137 v JSD</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr">
         <is>
           <t>🔴 červená</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B53" t="inlineStr">
         <is>
           <t>Nutno ověřit (popis/zařazení, Incoterm místo, hutní atest)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="15">
+    <mergeCell ref="B49:L49"/>
     <mergeCell ref="B4:L4"/>
-    <mergeCell ref="B26:L26"/>
+    <mergeCell ref="B50:L50"/>
+    <mergeCell ref="B53:L53"/>
     <mergeCell ref="B6:L6"/>
+    <mergeCell ref="B52:L52"/>
+    <mergeCell ref="B48:L48"/>
     <mergeCell ref="B7:L7"/>
     <mergeCell ref="B11:L11"/>
-    <mergeCell ref="B25:L25"/>
     <mergeCell ref="B3:L3"/>
     <mergeCell ref="B5:L5"/>
-    <mergeCell ref="B24:L24"/>
+    <mergeCell ref="B51:L51"/>
     <mergeCell ref="B10:L10"/>
-    <mergeCell ref="B22:L22"/>
-    <mergeCell ref="B23:L23"/>
     <mergeCell ref="B9:L9"/>
     <mergeCell ref="B8:L8"/>
   </mergeCells>
@@ -1186,1331 +2459,1331 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
+      <c r="A1" s="29" t="inlineStr">
         <is>
           <t>Odesílatel</t>
         </is>
       </c>
-      <c r="B1" s="22" t="inlineStr">
+      <c r="B1" s="29" t="inlineStr">
         <is>
           <t>Faktura</t>
         </is>
       </c>
-      <c r="C1" s="22" t="inlineStr">
+      <c r="C1" s="29" t="inlineStr">
         <is>
           <t>Part number</t>
         </is>
       </c>
-      <c r="D1" s="22" t="inlineStr">
+      <c r="D1" s="29" t="inlineStr">
         <is>
           <t>Popis (faktura, EN)</t>
         </is>
       </c>
-      <c r="E1" s="22" t="inlineStr">
+      <c r="E1" s="29" t="inlineStr">
         <is>
           <t>HS kód</t>
         </is>
       </c>
-      <c r="F1" s="22" t="inlineStr">
+      <c r="F1" s="29" t="inlineStr">
         <is>
           <t>Popis CZ (klient)</t>
         </is>
       </c>
-      <c r="G1" s="22" t="inlineStr">
+      <c r="G1" s="29" t="inlineStr">
         <is>
           <t>Množství (ks)</t>
         </is>
       </c>
-      <c r="H1" s="22" t="inlineStr">
+      <c r="H1" s="29" t="inlineStr">
         <is>
           <t>Čistá hm. (kg)</t>
         </is>
       </c>
-      <c r="I1" s="22" t="inlineStr">
+      <c r="I1" s="29" t="inlineStr">
         <is>
           <t>Hrubá hm. (kg)</t>
         </is>
       </c>
-      <c r="J1" s="22" t="inlineStr">
+      <c r="J1" s="29" t="inlineStr">
         <is>
           <t>Částka EUR</t>
         </is>
       </c>
-      <c r="K1" s="22" t="inlineStr">
+      <c r="K1" s="29" t="inlineStr">
         <is>
           <t>Zdroj</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
+      <c r="A2" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B2" s="23" t="inlineStr">
+      <c r="B2" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C2" s="23" t="inlineStr">
+      <c r="C2" s="30" t="inlineStr">
         <is>
           <t>IM-SW6515-VWCZ</t>
         </is>
       </c>
-      <c r="D2" s="23" t="inlineStr">
+      <c r="D2" s="30" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E2" s="24" t="inlineStr">
+      <c r="E2" s="31" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F2" s="23" t="inlineStr">
+      <c r="F2" s="30" t="inlineStr">
         <is>
           <t>Subwoofer</t>
         </is>
       </c>
-      <c r="G2" s="23" t="n">
+      <c r="G2" s="30" t="n">
         <v>540</v>
       </c>
-      <c r="H2" s="23" t="n">
+      <c r="H2" s="30" t="n">
         <v>313.2</v>
       </c>
-      <c r="I2" s="23" t="n">
+      <c r="I2" s="30" t="n">
         <v>350</v>
       </c>
-      <c r="J2" s="23" t="n">
+      <c r="J2" s="30" t="n">
         <v>2381.4</v>
       </c>
-      <c r="K2" s="23" t="inlineStr">
+      <c r="K2" s="30" t="inlineStr">
         <is>
           <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="23" t="inlineStr">
+      <c r="A3" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B3" s="23" t="inlineStr">
+      <c r="B3" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C3" s="23" t="inlineStr">
+      <c r="C3" s="30" t="inlineStr">
         <is>
           <t>IM-40138L-BMWCZ</t>
         </is>
       </c>
-      <c r="D3" s="23" t="inlineStr">
+      <c r="D3" s="30" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E3" s="24" t="inlineStr">
+      <c r="E3" s="31" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F3" s="23" t="inlineStr">
+      <c r="F3" s="30" t="inlineStr">
         <is>
           <t>Hotové reproduktory - ostatní</t>
         </is>
       </c>
-      <c r="G3" s="23" t="n">
+      <c r="G3" s="30" t="n">
         <v>540</v>
       </c>
-      <c r="H3" s="23" t="n">
+      <c r="H3" s="30" t="n">
         <v>253.8</v>
       </c>
-      <c r="I3" s="23" t="n">
+      <c r="I3" s="30" t="n">
         <v>270</v>
       </c>
-      <c r="J3" s="23" t="n">
+      <c r="J3" s="30" t="n">
         <v>4594.21</v>
       </c>
-      <c r="K3" s="23" t="inlineStr">
+      <c r="K3" s="30" t="inlineStr">
         <is>
           <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
+      <c r="A4" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B4" s="23" t="inlineStr">
+      <c r="B4" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C4" s="23" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>IM-65220G-BYCZ</t>
         </is>
       </c>
-      <c r="D4" s="23" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="31" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F4" s="23" t="inlineStr">
+      <c r="F4" s="30" t="inlineStr">
         <is>
           <t>Hotové reproduktory - ostatní</t>
         </is>
       </c>
-      <c r="G4" s="23" t="n">
+      <c r="G4" s="30" t="n">
         <v>360</v>
       </c>
-      <c r="H4" s="23" t="n">
+      <c r="H4" s="30" t="n">
         <v>270</v>
       </c>
-      <c r="I4" s="23" t="n">
+      <c r="I4" s="30" t="n">
         <v>308</v>
       </c>
-      <c r="J4" s="23" t="n">
+      <c r="J4" s="30" t="n">
         <v>3623.72</v>
       </c>
-      <c r="K4" s="23" t="inlineStr">
+      <c r="K4" s="30" t="inlineStr">
         <is>
           <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B5" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
         <is>
           <t>IM-SW6550-SKCZ</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D5" s="30" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="31" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F5" s="23" t="inlineStr">
+      <c r="F5" s="30" t="inlineStr">
         <is>
           <t>Subwoofer</t>
         </is>
       </c>
-      <c r="G5" s="23" t="n">
+      <c r="G5" s="30" t="n">
         <v>540</v>
       </c>
-      <c r="H5" s="23" t="n">
+      <c r="H5" s="30" t="n">
         <v>664.2</v>
       </c>
-      <c r="I5" s="23" t="n">
+      <c r="I5" s="30" t="n">
         <v>705.8200000000001</v>
       </c>
-      <c r="J5" s="23" t="n">
+      <c r="J5" s="30" t="n">
         <v>3607.2</v>
       </c>
-      <c r="K5" s="23" t="inlineStr">
+      <c r="K5" s="30" t="inlineStr">
         <is>
           <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B6" s="23" t="inlineStr">
+      <c r="B6" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="30" t="inlineStr">
         <is>
           <t>212-8061-1-CZ</t>
         </is>
       </c>
-      <c r="D6" s="23" t="inlineStr">
+      <c r="D6" s="30" t="inlineStr">
         <is>
           <t>Speaker component</t>
         </is>
       </c>
-      <c r="E6" s="24" t="inlineStr">
+      <c r="E6" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F6" s="23" t="inlineStr">
+      <c r="F6" s="30" t="inlineStr">
         <is>
           <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
         </is>
       </c>
-      <c r="G6" s="23" t="n">
+      <c r="G6" s="30" t="n">
         <v>4608</v>
       </c>
-      <c r="H6" s="23" t="n">
+      <c r="H6" s="30" t="n">
         <v>2211.84</v>
       </c>
-      <c r="I6" s="23" t="n">
+      <c r="I6" s="30" t="n">
         <v>2312</v>
       </c>
-      <c r="J6" s="23" t="n">
+      <c r="J6" s="30" t="n">
         <v>3170.3</v>
       </c>
-      <c r="K6" s="23" t="inlineStr">
+      <c r="K6" s="30" t="inlineStr">
         <is>
           <t>List1 ř.2 (obecná položka)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B7" s="23" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="30" t="inlineStr">
         <is>
           <t>IM-65386-BYCZ</t>
         </is>
       </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="30" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="E7" s="31" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F7" s="23" t="inlineStr">
+      <c r="F7" s="30" t="inlineStr">
         <is>
           <t>Hotové reproduktory - ostatní</t>
         </is>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="30" t="n">
         <v>240</v>
       </c>
-      <c r="H7" s="23" t="n">
+      <c r="H7" s="30" t="n">
         <v>175.2</v>
       </c>
-      <c r="I7" s="23" t="n">
+      <c r="I7" s="30" t="n">
         <v>195</v>
       </c>
-      <c r="J7" s="23" t="n">
+      <c r="J7" s="30" t="n">
         <v>2058.46</v>
       </c>
-      <c r="K7" s="23" t="inlineStr">
+      <c r="K7" s="30" t="inlineStr">
         <is>
           <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B8" s="23" t="inlineStr">
+      <c r="B8" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="30" t="inlineStr">
         <is>
           <t>IM-65387-BYCZ</t>
         </is>
       </c>
-      <c r="D8" s="23" t="inlineStr">
+      <c r="D8" s="30" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E8" s="24" t="inlineStr">
+      <c r="E8" s="31" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F8" s="23" t="inlineStr">
+      <c r="F8" s="30" t="inlineStr">
         <is>
           <t>Hotové reproduktory - ostatní</t>
         </is>
       </c>
-      <c r="G8" s="23" t="n">
+      <c r="G8" s="30" t="n">
         <v>180</v>
       </c>
-      <c r="H8" s="23" t="n">
+      <c r="H8" s="30" t="n">
         <v>133.2</v>
       </c>
-      <c r="I8" s="23" t="n">
+      <c r="I8" s="30" t="n">
         <v>152</v>
       </c>
-      <c r="J8" s="23" t="n">
+      <c r="J8" s="30" t="n">
         <v>1802.86</v>
       </c>
-      <c r="K8" s="23" t="inlineStr">
+      <c r="K8" s="30" t="inlineStr">
         <is>
           <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B9" s="23" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="30" t="inlineStr">
         <is>
           <t>IM-40137L-BMWCZ</t>
         </is>
       </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="30" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="31" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F9" s="23" t="inlineStr">
+      <c r="F9" s="30" t="inlineStr">
         <is>
           <t>Hotové reproduktory - ostatní</t>
         </is>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="30" t="n">
         <v>540</v>
       </c>
-      <c r="H9" s="23" t="n">
+      <c r="H9" s="30" t="n">
         <v>253.8</v>
       </c>
-      <c r="I9" s="23" t="n">
+      <c r="I9" s="30" t="n">
         <v>270</v>
       </c>
-      <c r="J9" s="23" t="n">
+      <c r="J9" s="30" t="n">
         <v>4199.09</v>
       </c>
-      <c r="K9" s="23" t="inlineStr">
+      <c r="K9" s="30" t="inlineStr">
         <is>
           <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B10" s="23" t="inlineStr">
+      <c r="B10" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="30" t="inlineStr">
         <is>
           <t>212-65424-CZ</t>
         </is>
       </c>
-      <c r="D10" s="23" t="inlineStr">
+      <c r="D10" s="30" t="inlineStr">
         <is>
           <t>Speaker component</t>
         </is>
       </c>
-      <c r="E10" s="24" t="inlineStr">
+      <c r="E10" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F10" s="23" t="inlineStr">
+      <c r="F10" s="30" t="inlineStr">
         <is>
           <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
         </is>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="30" t="n">
         <v>7680</v>
       </c>
-      <c r="H10" s="23" t="n">
+      <c r="H10" s="30" t="n">
         <v>1766.4</v>
       </c>
-      <c r="I10" s="23" t="n">
+      <c r="I10" s="30" t="n">
         <v>1797.6</v>
       </c>
-      <c r="J10" s="23" t="n">
+      <c r="J10" s="30" t="n">
         <v>1831.68</v>
       </c>
-      <c r="K10" s="23" t="inlineStr">
+      <c r="K10" s="30" t="inlineStr">
         <is>
           <t>List1 ř.2 (obecná položka)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="23" t="inlineStr">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B11" s="23" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="30" t="inlineStr">
         <is>
           <t>212-65581-CZ</t>
         </is>
       </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="D11" s="30" t="inlineStr">
         <is>
           <t>Speaker component</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F11" s="23" t="inlineStr">
+      <c r="F11" s="30" t="inlineStr">
         <is>
           <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
         </is>
       </c>
-      <c r="G11" s="23" t="n">
+      <c r="G11" s="30" t="n">
         <v>1053</v>
       </c>
-      <c r="H11" s="23" t="n">
+      <c r="H11" s="30" t="n">
         <v>452.79</v>
       </c>
-      <c r="I11" s="23" t="n">
+      <c r="I11" s="30" t="n">
         <v>489.32</v>
       </c>
-      <c r="J11" s="23" t="n">
+      <c r="J11" s="30" t="n">
         <v>694.98</v>
       </c>
-      <c r="K11" s="23" t="inlineStr">
+      <c r="K11" s="30" t="inlineStr">
         <is>
           <t>List1 ř.2 (obecná položka)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="30" t="inlineStr">
         <is>
           <t>040-65E4-C-CZ</t>
         </is>
       </c>
-      <c r="D12" s="23" t="inlineStr">
+      <c r="D12" s="30" t="inlineStr">
         <is>
           <t>Front plate</t>
         </is>
       </c>
-      <c r="E12" s="24" t="inlineStr">
+      <c r="E12" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F12" s="23" t="inlineStr">
+      <c r="F12" s="30" t="inlineStr">
         <is>
           <t>ocelová deska</t>
         </is>
       </c>
-      <c r="G12" s="23" t="n">
+      <c r="G12" s="30" t="n">
         <v>3000</v>
       </c>
-      <c r="H12" s="23" t="n">
+      <c r="H12" s="30" t="n">
         <v>222</v>
       </c>
-      <c r="I12" s="23" t="n">
+      <c r="I12" s="30" t="n">
         <v>225.43</v>
       </c>
-      <c r="J12" s="23" t="n">
+      <c r="J12" s="30" t="n">
         <v>309.9</v>
       </c>
-      <c r="K12" s="23" t="inlineStr">
+      <c r="K12" s="30" t="inlineStr">
         <is>
           <t>List2 ř.14 (+ dřívější JSD 85189000 00)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="23" t="inlineStr">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B13" s="23" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="30" t="inlineStr">
         <is>
           <t>210-50D3-17.5TCR-CZ</t>
         </is>
       </c>
-      <c r="D13" s="23" t="inlineStr">
+      <c r="D13" s="30" t="inlineStr">
         <is>
           <t>T-yoke</t>
         </is>
       </c>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F13" s="23" t="inlineStr">
+      <c r="F13" s="30" t="inlineStr">
         <is>
           <t>jádro magnetického obvodu</t>
         </is>
       </c>
-      <c r="G13" s="23" t="n">
+      <c r="G13" s="30" t="n">
         <v>17160</v>
       </c>
-      <c r="H13" s="23" t="n">
+      <c r="H13" s="30" t="n">
         <v>1115.4</v>
       </c>
-      <c r="I13" s="23" t="n">
+      <c r="I13" s="30" t="n">
         <v>1155.4</v>
       </c>
-      <c r="J13" s="23" t="n">
+      <c r="J13" s="30" t="n">
         <v>1395.11</v>
       </c>
-      <c r="K13" s="23" t="inlineStr">
+      <c r="K13" s="30" t="inlineStr">
         <is>
           <t>List2 ř.23</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="23" t="inlineStr">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B14" s="23" t="inlineStr">
+      <c r="B14" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="30" t="inlineStr">
         <is>
           <t>021-88E00-9-2-CZ</t>
         </is>
       </c>
-      <c r="D14" s="23" t="inlineStr">
+      <c r="D14" s="30" t="inlineStr">
         <is>
           <t>Spider</t>
         </is>
       </c>
-      <c r="E14" s="24" t="inlineStr">
+      <c r="E14" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F14" s="23" t="inlineStr">
+      <c r="F14" s="30" t="inlineStr">
         <is>
           <t>Středící membrána</t>
         </is>
       </c>
-      <c r="G14" s="23" t="n">
+      <c r="G14" s="30" t="n">
         <v>3000</v>
       </c>
-      <c r="H14" s="23" t="n">
+      <c r="H14" s="30" t="n">
         <v>4.5</v>
       </c>
-      <c r="I14" s="23" t="n">
+      <c r="I14" s="30" t="n">
         <v>9.5</v>
       </c>
-      <c r="J14" s="23" t="n">
+      <c r="J14" s="30" t="n">
         <v>282.6</v>
       </c>
-      <c r="K14" s="23" t="inlineStr">
+      <c r="K14" s="30" t="inlineStr">
         <is>
           <t>List2 ř.7</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="23" t="inlineStr">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B15" s="23" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="30" t="inlineStr">
         <is>
           <t>142-530H10-10H-CZ</t>
         </is>
       </c>
-      <c r="D15" s="23" t="inlineStr">
+      <c r="D15" s="30" t="inlineStr">
         <is>
           <t>Gasket</t>
         </is>
       </c>
-      <c r="E15" s="24" t="inlineStr">
+      <c r="E15" s="31" t="inlineStr">
         <is>
           <t>3926909790</t>
         </is>
       </c>
-      <c r="F15" s="23" t="inlineStr">
+      <c r="F15" s="30" t="inlineStr">
         <is>
           <t>plastové těsnění</t>
         </is>
       </c>
-      <c r="G15" s="23" t="n">
+      <c r="G15" s="30" t="n">
         <v>3000</v>
       </c>
-      <c r="H15" s="23" t="n">
+      <c r="H15" s="30" t="n">
         <v>22.5</v>
       </c>
-      <c r="I15" s="23" t="n">
+      <c r="I15" s="30" t="n">
         <v>27.5</v>
       </c>
-      <c r="J15" s="23" t="n">
+      <c r="J15" s="30" t="n">
         <v>126</v>
       </c>
-      <c r="K15" s="23" t="inlineStr">
+      <c r="K15" s="30" t="inlineStr">
         <is>
           <t>List2 ř.50 (39269097); díly 142-*, ne 143-* (gumové)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B16" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="30" t="inlineStr">
         <is>
           <t>142-65580-3A-CZ</t>
         </is>
       </c>
-      <c r="D16" s="23" t="inlineStr">
+      <c r="D16" s="30" t="inlineStr">
         <is>
           <t>Gasket</t>
         </is>
       </c>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="E16" s="31" t="inlineStr">
         <is>
           <t>3926909790</t>
         </is>
       </c>
-      <c r="F16" s="23" t="inlineStr">
+      <c r="F16" s="30" t="inlineStr">
         <is>
           <t>plastové těsnění</t>
         </is>
       </c>
-      <c r="G16" s="23" t="n">
+      <c r="G16" s="30" t="n">
         <v>3000</v>
       </c>
-      <c r="H16" s="23" t="n">
+      <c r="H16" s="30" t="n">
         <v>22.5</v>
       </c>
-      <c r="I16" s="23" t="n">
+      <c r="I16" s="30" t="n">
         <v>27.5</v>
       </c>
-      <c r="J16" s="23" t="n">
+      <c r="J16" s="30" t="n">
         <v>144</v>
       </c>
-      <c r="K16" s="23" t="inlineStr">
+      <c r="K16" s="30" t="inlineStr">
         <is>
           <t>List2 ř.50 (39269097); díly 142-*, ne 143-* (gumové)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="30" t="inlineStr">
         <is>
           <t>181-40133-1SN-CZ</t>
         </is>
       </c>
-      <c r="D17" s="23" t="inlineStr">
+      <c r="D17" s="30" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E17" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F17" s="23" t="inlineStr">
+      <c r="F17" s="30" t="inlineStr">
         <is>
           <t>Terminál</t>
         </is>
       </c>
-      <c r="G17" s="23" t="n">
+      <c r="G17" s="30" t="n">
         <v>150000</v>
       </c>
-      <c r="H17" s="23" t="n">
+      <c r="H17" s="30" t="n">
         <v>75</v>
       </c>
-      <c r="I17" s="23" t="n">
+      <c r="I17" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="23" t="n">
+      <c r="J17" s="30" t="n">
         <v>1905</v>
       </c>
-      <c r="K17" s="23" t="inlineStr">
+      <c r="K17" s="30" t="inlineStr">
         <is>
           <t>List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="23" t="inlineStr">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B18" s="23" t="inlineStr">
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="30" t="inlineStr">
         <is>
           <t>181-40133-2SN-CZ</t>
         </is>
       </c>
-      <c r="D18" s="23" t="inlineStr">
+      <c r="D18" s="30" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="E18" s="24" t="inlineStr">
+      <c r="E18" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F18" s="23" t="inlineStr">
+      <c r="F18" s="30" t="inlineStr">
         <is>
           <t>Terminál</t>
         </is>
       </c>
-      <c r="G18" s="23" t="n">
+      <c r="G18" s="30" t="n">
         <v>150000</v>
       </c>
-      <c r="H18" s="23" t="n">
+      <c r="H18" s="30" t="n">
         <v>75</v>
       </c>
-      <c r="I18" s="23" t="n">
+      <c r="I18" s="30" t="n">
         <v>80</v>
       </c>
-      <c r="J18" s="23" t="n">
+      <c r="J18" s="30" t="n">
         <v>1905</v>
       </c>
-      <c r="K18" s="23" t="inlineStr">
+      <c r="K18" s="30" t="inlineStr">
         <is>
           <t>List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="23" t="inlineStr">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="30" t="inlineStr">
         <is>
           <t>029-2513-AL-CZ</t>
         </is>
       </c>
-      <c r="D19" s="23" t="inlineStr">
+      <c r="D19" s="30" t="inlineStr">
         <is>
           <t>Nut</t>
         </is>
       </c>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="E19" s="31" t="inlineStr">
         <is>
           <t>7318169290</t>
         </is>
       </c>
-      <c r="F19" s="23" t="inlineStr">
+      <c r="F19" s="30" t="inlineStr">
         <is>
           <t>Nut</t>
         </is>
       </c>
-      <c r="G19" s="23" t="n">
+      <c r="G19" s="30" t="n">
         <v>100000</v>
       </c>
-      <c r="H19" s="23" t="n">
+      <c r="H19" s="30" t="n">
         <v>166.5</v>
       </c>
-      <c r="I19" s="23" t="n">
+      <c r="I19" s="30" t="n">
         <v>172.5</v>
       </c>
-      <c r="J19" s="23" t="n">
+      <c r="J19" s="30" t="n">
         <v>7000</v>
       </c>
-      <c r="K19" s="23" t="inlineStr">
+      <c r="K19" s="30" t="inlineStr">
         <is>
           <t>List2 ř.202 ('tohle řadíme pod 7318169290') – bez CZ popisu</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="23" t="inlineStr">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="30" t="inlineStr">
         <is>
           <t>140-35D14-44XP1-CZ</t>
         </is>
       </c>
-      <c r="D20" s="23" t="inlineStr">
+      <c r="D20" s="30" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E20" s="24" t="inlineStr">
+      <c r="E20" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F20" s="23" t="inlineStr">
+      <c r="F20" s="30" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G20" s="23" t="n">
+      <c r="G20" s="30" t="n">
         <v>34000</v>
       </c>
-      <c r="H20" s="23" t="n">
+      <c r="H20" s="30" t="n">
         <v>68</v>
       </c>
-      <c r="I20" s="23" t="n">
+      <c r="I20" s="30" t="n">
         <v>130</v>
       </c>
-      <c r="J20" s="23" t="n">
+      <c r="J20" s="30" t="n">
         <v>12437.2</v>
       </c>
-      <c r="K20" s="23" t="inlineStr">
+      <c r="K20" s="30" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="23" t="inlineStr">
+      <c r="A21" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B21" s="23" t="inlineStr">
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="30" t="inlineStr">
         <is>
           <t>015-S753215-Y30-KS-CZ</t>
         </is>
       </c>
-      <c r="D21" s="23" t="inlineStr">
+      <c r="D21" s="30" t="inlineStr">
         <is>
           <t>Speaker components</t>
         </is>
       </c>
-      <c r="E21" s="24" t="inlineStr">
+      <c r="E21" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F21" s="23" t="inlineStr">
+      <c r="F21" s="30" t="inlineStr">
         <is>
           <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
         </is>
       </c>
-      <c r="G21" s="23" t="n">
+      <c r="G21" s="30" t="n">
         <v>21600</v>
       </c>
-      <c r="H21" s="23" t="n">
+      <c r="H21" s="30" t="n">
         <v>5616</v>
       </c>
-      <c r="I21" s="23" t="n">
+      <c r="I21" s="30" t="n">
         <v>5736</v>
       </c>
-      <c r="J21" s="23" t="n">
+      <c r="J21" s="30" t="n">
         <v>5978.88</v>
       </c>
-      <c r="K21" s="23" t="inlineStr">
+      <c r="K21" s="30" t="inlineStr">
         <is>
           <t>List1 ř.2 (obecná položka)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="30" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B22" s="23" t="inlineStr">
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="30" t="inlineStr">
         <is>
           <t>210-66E2-24.5TCR-1-CZ</t>
         </is>
       </c>
-      <c r="D22" s="23" t="inlineStr">
+      <c r="D22" s="30" t="inlineStr">
         <is>
           <t>T-yoke</t>
         </is>
       </c>
-      <c r="E22" s="24" t="inlineStr">
+      <c r="E22" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F22" s="23" t="inlineStr">
+      <c r="F22" s="30" t="inlineStr">
         <is>
           <t>jádro magnetického obvodu</t>
         </is>
       </c>
-      <c r="G22" s="23" t="n">
+      <c r="G22" s="30" t="n">
         <v>42840</v>
       </c>
-      <c r="H22" s="23" t="n">
+      <c r="H22" s="30" t="n">
         <v>6897.24</v>
       </c>
-      <c r="I22" s="23" t="n">
+      <c r="I22" s="30" t="n">
         <v>7037.24</v>
       </c>
-      <c r="J22" s="23" t="n">
+      <c r="J22" s="30" t="n">
         <v>8186.72</v>
       </c>
-      <c r="K22" s="23" t="inlineStr">
+      <c r="K22" s="30" t="inlineStr">
         <is>
           <t>List2 ř.23</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="23" t="inlineStr">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B23" s="23" t="inlineStr">
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="30" t="inlineStr">
         <is>
           <t>140-65D24-179X-CZ</t>
         </is>
       </c>
-      <c r="D23" s="23" t="inlineStr">
+      <c r="D23" s="30" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="E23" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F23" s="23" t="inlineStr">
+      <c r="F23" s="30" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G23" s="23" t="n">
+      <c r="G23" s="30" t="n">
         <v>17280</v>
       </c>
-      <c r="H23" s="23" t="n">
+      <c r="H23" s="30" t="n">
         <v>240</v>
       </c>
-      <c r="I23" s="23" t="n">
+      <c r="I23" s="30" t="n">
         <v>373.33</v>
       </c>
-      <c r="J23" s="23" t="n">
+      <c r="J23" s="30" t="n">
         <v>4397.76</v>
       </c>
-      <c r="K23" s="23" t="inlineStr">
+      <c r="K23" s="30" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="23" t="inlineStr">
+      <c r="A24" s="30" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B24" s="23" t="inlineStr">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C24" s="23" t="inlineStr">
+      <c r="C24" s="30" t="inlineStr">
         <is>
           <t>140-80I27-42X-CZ</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D24" s="30" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E24" s="24" t="inlineStr">
+      <c r="E24" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F24" s="23" t="inlineStr">
+      <c r="F24" s="30" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G24" s="23" t="n">
+      <c r="G24" s="30" t="n">
         <v>24000</v>
       </c>
-      <c r="H24" s="23" t="n">
+      <c r="H24" s="30" t="n">
         <v>612</v>
       </c>
-      <c r="I24" s="23" t="n">
+      <c r="I24" s="30" t="n">
         <v>810</v>
       </c>
-      <c r="J24" s="23" t="n">
+      <c r="J24" s="30" t="n">
         <v>12026.4</v>
       </c>
-      <c r="K24" s="23" t="inlineStr">
+      <c r="K24" s="30" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="23" t="inlineStr">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B25" s="23" t="inlineStr">
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C25" s="23" t="inlineStr">
+      <c r="C25" s="30" t="inlineStr">
         <is>
           <t>160-B29-H-CZ</t>
         </is>
       </c>
-      <c r="D25" s="23" t="inlineStr">
+      <c r="D25" s="30" t="inlineStr">
         <is>
           <t>Dust cap</t>
         </is>
       </c>
-      <c r="E25" s="24" t="inlineStr">
+      <c r="E25" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F25" s="23" t="inlineStr">
+      <c r="F25" s="30" t="inlineStr">
         <is>
           <t>Kopulka= krycí vložka</t>
         </is>
       </c>
-      <c r="G25" s="23" t="n">
+      <c r="G25" s="30" t="n">
         <v>52000</v>
       </c>
-      <c r="H25" s="23" t="n">
+      <c r="H25" s="30" t="n">
         <v>12.6</v>
       </c>
-      <c r="I25" s="23" t="n">
+      <c r="I25" s="30" t="n">
         <v>17.1</v>
       </c>
-      <c r="J25" s="23" t="n">
+      <c r="J25" s="30" t="n">
         <v>8034</v>
       </c>
-      <c r="K25" s="23" t="inlineStr">
+      <c r="K25" s="30" t="inlineStr">
         <is>
           <t>List2 ř.9 (uvedeno 8518 9000 99)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="23" t="inlineStr">
+      <c r="A26" s="30" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B26" s="23" t="inlineStr">
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C26" s="23" t="inlineStr">
+      <c r="C26" s="30" t="inlineStr">
         <is>
           <t>140-65E22-203X-CZ</t>
         </is>
       </c>
-      <c r="D26" s="23" t="inlineStr">
+      <c r="D26" s="30" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E26" s="24" t="inlineStr">
+      <c r="E26" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F26" s="23" t="inlineStr">
+      <c r="F26" s="30" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G26" s="23" t="n">
+      <c r="G26" s="30" t="n">
         <v>3000</v>
       </c>
-      <c r="H26" s="23" t="n">
+      <c r="H26" s="30" t="n">
         <v>25.91</v>
       </c>
-      <c r="I26" s="23" t="n">
+      <c r="I26" s="30" t="n">
         <v>39.36</v>
       </c>
-      <c r="J26" s="23" t="n">
+      <c r="J26" s="30" t="n">
         <v>895.5</v>
       </c>
-      <c r="K26" s="23" t="inlineStr">
+      <c r="K26" s="30" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="23" t="inlineStr">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B27" s="23" t="inlineStr">
+      <c r="B27" s="30" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C27" s="23" t="inlineStr">
+      <c r="C27" s="30" t="inlineStr">
         <is>
           <t>140-40E17-72XC-CZ</t>
         </is>
       </c>
-      <c r="D27" s="23" t="inlineStr">
+      <c r="D27" s="30" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E27" s="24" t="inlineStr">
+      <c r="E27" s="31" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F27" s="23" t="inlineStr">
+      <c r="F27" s="30" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G27" s="23" t="n">
+      <c r="G27" s="30" t="n">
         <v>14400</v>
       </c>
-      <c r="H27" s="23" t="n">
+      <c r="H27" s="30" t="n">
         <v>86.40000000000001</v>
       </c>
-      <c r="I27" s="23" t="n">
+      <c r="I27" s="30" t="n">
         <v>101.34</v>
       </c>
-      <c r="J27" s="23" t="n">
+      <c r="J27" s="30" t="n">
         <v>4883.04</v>
       </c>
-      <c r="K27" s="23" t="inlineStr">
+      <c r="K27" s="30" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
@@ -2534,189 +3807,189 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="25" t="inlineStr">
+      <c r="A1" s="32" t="inlineStr">
         <is>
           <t>PREFERENČNÍ VĚTA (COO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="26" t="inlineStr">
+      <c r="A2" s="33" t="inlineStr">
         <is>
           <t>Na žádné ze 3 faktur NENÍ preferenční věta. Země původu Čína → bez preferencí, platí standardní clo (8518 90 00 0 %, 8518 29 3 %*, 3926 90 97 6,5 %, 7318 16 3,7 %).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="25" t="inlineStr">
+      <c r="A3" s="32" t="inlineStr">
         <is>
           <t>REX ČÍSLO</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="26" t="inlineStr">
+      <c r="A4" s="33" t="inlineStr">
         <is>
           <t>REX číslo NENÍ uvedeno na žádné faktuře (CZ20260904, CZ20260904-1, CZ20260904-2).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="25" t="inlineStr">
+      <c r="A5" s="32" t="inlineStr">
         <is>
           <t>CBAM – příjemce Sonavox Technology CZ s.r.o.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="33" t="inlineStr">
         <is>
           <t>CBAM HS kód: 7318169290 (matice, 166,5 kg NW, odesílatel Suzhou Sonavox International Trading).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
+      <c r="A7" s="33" t="inlineStr">
         <is>
           <t>Registr reference/CBAM_receivers_CZ.xlsx: 'Sonavox Technology CZ s.r.o.' NALEZEN → Y KÓD = Y137 (do 50 t ročně). Povolení: –, podaná žádost: –, datum vydání: neuvedeno.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="inlineStr">
+      <c r="A8" s="34" t="inlineStr">
         <is>
           <t>⚠ NESOULAD EORI: registr uvádí EORI CZ62908227, ale ref. soubor klienta uvádí 'EORI=DIČ=CZ28632389'. CZ62908227 je na FCR uvedeno jako VAT zasílatele (Maurice Ward &amp; Co.) → pravděpodobně chyba v registru, ověřit a opravit.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="26" t="inlineStr">
+      <c r="A9" s="33" t="inlineStr">
         <is>
           <t>Není to firma mimo EU na sdíleném účtu CBAM-CZ-2025-QGM67089385721.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="25" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>MELT AND POUR (země tavby a odlití)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="inlineStr">
+      <c r="A11" s="34" t="inlineStr">
         <is>
           <t>CHYBÍ: v dokladech není hutní atest (mill test certificate) ani země tavby a odlití. Týká se ocelových matic 7318169290 (029-2513-AL-CZ, 100 000 ks, 166,5 kg) → vyžádat hutní atest před proclením.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="26" t="inlineStr">
+      <c r="A12" s="33" t="inlineStr">
         <is>
           <t>Ocelové díly zařazené jako díly reproduktorů 8518 90 00 (Front plate 'ocelová deska' 222 kg, T-yoke 'jádro magnetického obvodu' 8 012,64 kg) – mimo kap. 72/73, ale ocelové; hutní atest také není k dispozici – doporučuji vyžádat.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="26" t="inlineStr">
+      <c r="A13" s="33" t="inlineStr">
         <is>
           <t>Pokud se potvrdí, že matice jsou hliníkové ('AL'), melt and pour (ocel) se na ně nevztahuje, ale CBAM ano (7616 10 00).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="25" t="inlineStr">
+      <c r="A14" s="32" t="inlineStr">
         <is>
           <t>ANTIDUMPING</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="26" t="inlineStr">
+      <c r="A15" s="33" t="inlineStr">
         <is>
           <t>Žádná položka podle aktuálního zařazení nepodléhá antidumpingu. Matice 7318 16 nejsou v rozsahu AD cla na spojovací prvky z CN (šrouby 7318 15 – 86,5 % dle ref. klienta – v zásilce nejsou). Ověřit při podání JSD.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="25" t="inlineStr">
+      <c r="A16" s="32" t="inlineStr">
         <is>
           <t>INCOTERM</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="inlineStr">
+      <c r="A17" s="34" t="inlineStr">
         <is>
           <t>Faktury: 'Terms of Payment: FOB' – BEZ pojmenovaného místa. FCR: místo převzetí Wuhan, Hubei; FREIGHT COLLECT. FOB je námořní doložka, zde železnice → doplnit místo (FOB Wuhan? / Suzhou?) od klienta.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="25" t="inlineStr">
+      <c r="A18" s="32" t="inlineStr">
         <is>
           <t>HODNOTA – 'Total'</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="26" t="inlineStr">
+      <c r="A19" s="33" t="inlineStr">
         <is>
           <t>CZ20260904-1 (Sonavox Electronics): Total Amount = 27 963,90 EUR ✓.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="inlineStr">
+      <c r="A20" s="34" t="inlineStr">
         <is>
           <t>CZ20260904 (Sonavox International Trading) a CZ20260904-2 (Yanlong): řádek 'Total Amount' je PRÁZDNÝ; 'Total :' je jen u množství. Použit Sub Total 39 670,41 a 30 236,70 EUR (Duty/Freight/Insurance prázdné, bez slevy) – potvrdit.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="25" t="inlineStr">
+      <c r="A21" s="32" t="inlineStr">
         <is>
           <t>CCT/VPV KN</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="26" t="inlineStr">
+      <c r="A22" s="33" t="inlineStr">
         <is>
           <t>Pravidlo CCT/VPV KN nebylo použito – všechny položky mají HS kód v referenčním souboru klienta 'Celní zařazení obvyklých položek Sonavox'. Faktury samy HS kódy neuvádějí; CIM uvádí pro vše 8518900000.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="25" t="inlineStr">
+      <c r="A23" s="32" t="inlineStr">
         <is>
           <t>ZAŘAZENÍ K OVĚŘENÍ</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="26" t="inlineStr">
+      <c r="A24" s="33" t="inlineStr">
         <is>
           <t>Gasket (142-*) – plast 3926909790 vs. pryž 4016 vs. pěna 3921; materiál nepotvrzen.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="26" t="inlineStr">
+      <c r="A25" s="33" t="inlineStr">
         <is>
           <t>Nut (029-2513-AL-CZ) – klient nemá český popis; 'AL' → možná hliník (7616 10 00).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="A26" s="33" t="inlineStr">
         <is>
           <t>Speaker components 015-S753215-Y30-KS-CZ (5 616 kg) – 'Y30' = feritová třída → spíše magnet (8505 19 dle Pozn. 2a tř. XVI) než 8518 90 00 – případně konzultovat s customs.tariff@mauriceward.com.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="26" t="inlineStr">
+      <c r="A27" s="33" t="inlineStr">
         <is>
           <t>Car speakers – 8518290090 (poslední poznámka klienta) vs. 8518 29 95 (List1). *Sazba 3 % dle List1 – ověřit v TARIC.</t>
         </is>

</xml_diff>

<commit_message>
Sonavox CICU2064021: use specific Czech item names
Replace the generic tariff wording ("Hotové reproduktory - ostatní",
"Komponenty ... - Ostatní ...") with the item names from the client's
reference file (magnetický obvod, Hotové reproduktory, ocelová deska
(přední deska), ...). Items with no Czech name in the client file
(Feritový magnet, Matice) are marked with a warning and red fill.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TDfNjvRhvE2vaNKifmBYbR
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_Sonavox_CICU2064021.xlsx
+++ b/output/HS_Code_Summary_Sonavox_CICU2064021.xlsx
@@ -105,7 +105,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,6 +148,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -766,8 +769,8 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>• Subwoofer  ← faktura: "Car Speaker" – 1 080 ks | NW 977,400 kg | GW 1 055,820 kg | 5 988,60 EUR
-• Hotové reproduktory - ostatní  ← faktura: "Car Speaker" – 1 860 ks | NW 1 086,000 kg | GW 1 195,000 kg | 16 278,34 EUR</t>
+          <t>• Subwoofer
+• Hotové reproduktory</t>
         </is>
       </c>
       <c r="E14" s="8" t="n">
@@ -790,7 +793,7 @@
       <c r="J14" s="11" t="inlineStr"/>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090') | List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+          <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090') | List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
       <c r="L14" s="11" t="inlineStr">
@@ -869,7 +872,7 @@
       </c>
       <c r="D16" s="12" t="inlineStr">
         <is>
-          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+          <t>Hotové reproduktory  ← faktura: "Car Speaker"</t>
         </is>
       </c>
       <c r="E16" s="14" t="n">
@@ -888,7 +891,7 @@
       <c r="J16" s="12" t="inlineStr"/>
       <c r="K16" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
       <c r="L16" s="12" t="inlineStr">
@@ -916,7 +919,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+          <t>Hotové reproduktory  ← faktura: "Car Speaker"</t>
         </is>
       </c>
       <c r="E17" s="14" t="n">
@@ -935,7 +938,7 @@
       <c r="J17" s="12" t="inlineStr"/>
       <c r="K17" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
       <c r="L17" s="12" t="inlineStr">
@@ -1010,7 +1013,7 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+          <t>Hotové reproduktory  ← faktura: "Car Speaker"</t>
         </is>
       </c>
       <c r="E19" s="14" t="n">
@@ -1029,7 +1032,7 @@
       <c r="J19" s="12" t="inlineStr"/>
       <c r="K19" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
       <c r="L19" s="12" t="inlineStr">
@@ -1057,7 +1060,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+          <t>Hotové reproduktory  ← faktura: "Car Speaker"</t>
         </is>
       </c>
       <c r="E20" s="14" t="n">
@@ -1076,7 +1079,7 @@
       <c r="J20" s="12" t="inlineStr"/>
       <c r="K20" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
       <c r="L20" s="12" t="inlineStr">
@@ -1104,7 +1107,7 @@
       </c>
       <c r="D21" s="12" t="inlineStr">
         <is>
-          <t>Hotové reproduktory - ostatní  ← faktura: "Car Speaker"</t>
+          <t>Hotové reproduktory  ← faktura: "Car Speaker"</t>
         </is>
       </c>
       <c r="E21" s="14" t="n">
@@ -1123,7 +1126,7 @@
       <c r="J21" s="12" t="inlineStr"/>
       <c r="K21" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
       <c r="L21" s="12" t="inlineStr">
@@ -1151,7 +1154,7 @@
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
-          <t>• Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component" – 13 341 ks | NW 4 431,030 kg | GW 4 598,920 kg | 5 696,96 EUR</t>
+          <t>• magnetický obvod</t>
         </is>
       </c>
       <c r="E22" s="8" t="n">
@@ -1174,7 +1177,7 @@
       <c r="J22" s="11" t="inlineStr"/>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>List1 ř.2 (obecná položka)</t>
+          <t>List2 ř.37 'magnetický obvod'; řada 212-* = magnetový obvod (List1 ř.3: 212-65163-CZ)</t>
         </is>
       </c>
       <c r="L22" s="11" t="inlineStr">
@@ -1184,7 +1187,7 @@
       </c>
       <c r="M22" s="11" t="inlineStr">
         <is>
-          <t>Díly 212-* = rodina magnetických obvodů (List1 ř.3: 212-65163-CZ neodym → 8518 9000 30). Pokud jsou neodymové, ověřit podpoložku 30.</t>
+          <t>Faktura uvádí jen 'Speaker component'; díly 212-* = řada magnetových obvodů (List1 ř.3: 212-65163-CZ) → 'magnetický obvod'. Pokud neodymové → ověřit 8518 9000 30.</t>
         </is>
       </c>
     </row>
@@ -1206,7 +1209,7 @@
       </c>
       <c r="D23" s="12" t="inlineStr">
         <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component"</t>
+          <t>magnetický obvod  ← faktura: "Speaker component"</t>
         </is>
       </c>
       <c r="E23" s="14" t="n">
@@ -1225,7 +1228,7 @@
       <c r="J23" s="12" t="inlineStr"/>
       <c r="K23" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.2 (obecná položka)</t>
+          <t>List2 ř.37 'magnetický obvod'; řada 212-* = magnetový obvod (List1 ř.3: 212-65163-CZ)</t>
         </is>
       </c>
       <c r="L23" s="12" t="inlineStr">
@@ -1253,7 +1256,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component"</t>
+          <t>magnetický obvod  ← faktura: "Speaker component"</t>
         </is>
       </c>
       <c r="E24" s="14" t="n">
@@ -1272,7 +1275,7 @@
       <c r="J24" s="12" t="inlineStr"/>
       <c r="K24" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.2 (obecná položka)</t>
+          <t>List2 ř.37 'magnetický obvod'; řada 212-* = magnetový obvod (List1 ř.3: 212-65163-CZ)</t>
         </is>
       </c>
       <c r="L24" s="12" t="inlineStr">
@@ -1300,7 +1303,7 @@
       </c>
       <c r="D25" s="12" t="inlineStr">
         <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker component"</t>
+          <t>magnetický obvod  ← faktura: "Speaker component"</t>
         </is>
       </c>
       <c r="E25" s="14" t="n">
@@ -1319,7 +1322,7 @@
       <c r="J25" s="12" t="inlineStr"/>
       <c r="K25" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.2 (obecná položka)</t>
+          <t>List2 ř.37 'magnetický obvod'; řada 212-* = magnetový obvod (List1 ř.3: 212-65163-CZ)</t>
         </is>
       </c>
       <c r="L25" s="12" t="inlineStr">
@@ -1345,14 +1348,14 @@
           <t>8518900000</t>
         </is>
       </c>
-      <c r="D26" s="6" t="inlineStr">
-        <is>
-          <t>• ocelová deska  ← faktura: "Front plate" – 3 000 ks | NW 222,000 kg | GW 225,430 kg | 309,90 EUR
-• jádro magnetického obvodu  ← faktura: "T-yoke" – 60 000 ks | NW 8 012,640 kg | GW 8 192,640 kg | 9 581,83 EUR
-• Středící membrána  ← faktura: "Spider" – 3 000 ks | NW 4,500 kg | GW 9,500 kg | 282,60 EUR
-• Terminál  ← faktura: "Terminal" – 300 000 ks | NW 150,000 kg | GW 160,000 kg | 3 810,00 EUR
-• Membrána s vlnkou  ← faktura: "Cone" – 34 000 ks | NW 68,000 kg | GW 130,000 kg | 12 437,20 EUR
-• Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker components" – 21 600 ks | NW 5 616,000 kg | GW 5 736,000 kg | 5 978,88 EUR</t>
+      <c r="D26" s="17" t="inlineStr">
+        <is>
+          <t>• ocelová deska (přední deska)
+• jádro magnetického obvodu
+• Středící membrána
+• Terminál
+• Membrána s vlnkou
+• Feritový magnet ⚠</t>
         </is>
       </c>
       <c r="E26" s="8" t="n">
@@ -1375,7 +1378,7 @@
       <c r="J26" s="11" t="inlineStr"/>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>List2 ř.14 (+ dřívější JSD 85189000 00) | List2 ř.23 | List2 ř.7 | List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ) | List2 ř.8 / List1 ř.4 | List1 ř.2 (obecná položka)</t>
+          <t>List2 ř.14 (+ dřívější JSD 85189000 00) | List2 ř.23 | List2 ř.7 | List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ) | List2 ř.8 / List1 ř.4 | List2 ř.29 'MAGNET' 8518900000 – CZ popis v ref. souboru NENÍ (S753215 = kroužek 75×32×15 mm, Y30 = ferit)</t>
         </is>
       </c>
       <c r="L26" s="11" t="inlineStr">
@@ -1385,7 +1388,7 @@
       </c>
       <c r="M26" s="11" t="inlineStr">
         <is>
-          <t>Front plate: List1/List2 uvádí 8518900090, ale dřívější JSD klienta (přední deska) = 85189000 00 – '90' byla čistá hmotnost. 015-S753215-Y30-KS-CZ: 'Y30' = třída feritu → pravděpodobně feritový magnet; dle Pozn. 2a k tř. XVI by mohl patřit pod 8505 19 – klient řadí magnety pod 8518900000 (List2 'MAGNET'). Ocelové díly (front plate, T-yoke) – viz melt and pour.</t>
+          <t>Front plate: List1/List2 uvádí 8518900090, ale dřívější JSD klienta (přední deska) = 85189000 00 – '90' byla čistá hmotnost. 015-S753215-Y30-KS-CZ = feritový magnet (kroužek 75×32×15 mm, Y30; 260 g/ks sedí) – český popis v ref. souboru klienta NENÍ, doplněn námi; dle Pozn. 2a k tř. XVI by mohl patřit pod 8505 19 – klient řadí magnety pod 8518900000 (List2 'MAGNET'). Ocelové díly (front plate, T-yoke) – viz melt and pour.</t>
         </is>
       </c>
     </row>
@@ -1407,7 +1410,7 @@
       </c>
       <c r="D27" s="12" t="inlineStr">
         <is>
-          <t>ocelová deska  ← faktura: "Front plate"</t>
+          <t>ocelová deska (přední deska)  ← faktura: "Front plate"</t>
         </is>
       </c>
       <c r="E27" s="14" t="n">
@@ -1687,9 +1690,9 @@
           <t>8518900000</t>
         </is>
       </c>
-      <c r="D33" s="12" t="inlineStr">
-        <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže  ← faktura: "Speaker components"</t>
+      <c r="D33" s="18" t="inlineStr">
+        <is>
+          <t>Feritový magnet ⚠ (CZ popis není v ref. souboru klienta)  ← faktura: "Speaker components"</t>
         </is>
       </c>
       <c r="E33" s="14" t="n">
@@ -1708,7 +1711,7 @@
       <c r="J33" s="12" t="inlineStr"/>
       <c r="K33" s="12" t="inlineStr">
         <is>
-          <t>List1 ř.2 (obecná položka)</t>
+          <t>List2 ř.29 'MAGNET' 8518900000 – CZ popis v ref. souboru NENÍ (S753215 = kroužek 75×32×15 mm, Y30 = ferit)</t>
         </is>
       </c>
       <c r="L33" s="12" t="inlineStr">
@@ -1783,7 +1786,7 @@
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>• plastové těsnění  ← faktura: "Gasket" – 6 000 ks | NW 45,000 kg | GW 55,000 kg | 270,00 EUR</t>
+          <t>• plastové těsnění</t>
         </is>
       </c>
       <c r="E35" s="8" t="n">
@@ -1915,59 +1918,59 @@
       <c r="M37" s="12" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="18" t="inlineStr">
+      <c r="A38" s="19" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B38" s="18" t="inlineStr">
+      <c r="B38" s="19" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C38" s="19" t="inlineStr">
+      <c r="C38" s="20" t="inlineStr">
         <is>
           <t>7318169290</t>
         </is>
       </c>
       <c r="D38" s="17" t="inlineStr">
         <is>
-          <t>• Nut  ← faktura: "Nut" – 100 000 ks | NW 166,500 kg | GW 172,500 kg | 7 000,00 EUR</t>
-        </is>
-      </c>
-      <c r="E38" s="20" t="n">
+          <t>• Matice ⚠</t>
+        </is>
+      </c>
+      <c r="E38" s="21" t="n">
         <v>100000</v>
       </c>
-      <c r="F38" s="21" t="n">
+      <c r="F38" s="22" t="n">
         <v>166.5</v>
       </c>
-      <c r="G38" s="21" t="n">
+      <c r="G38" s="22" t="n">
         <v>172.5</v>
       </c>
-      <c r="H38" s="22" t="n">
+      <c r="H38" s="23" t="n">
         <v>7000</v>
       </c>
-      <c r="I38" s="23" t="inlineStr">
+      <c r="I38" s="24" t="inlineStr">
         <is>
           <t>3,7 %</t>
         </is>
       </c>
-      <c r="J38" s="23" t="inlineStr">
+      <c r="J38" s="24" t="inlineStr">
         <is>
           <t>CBAM, MELT&amp;POUR</t>
         </is>
       </c>
-      <c r="K38" s="23" t="inlineStr">
+      <c r="K38" s="24" t="inlineStr">
         <is>
           <t>List2 ř.202 ('tohle řadíme pod 7318169290') – bez CZ popisu</t>
         </is>
       </c>
-      <c r="L38" s="23" t="inlineStr">
+      <c r="L38" s="24" t="inlineStr">
         <is>
           <t>029-2513-AL-CZ</t>
         </is>
       </c>
-      <c r="M38" s="23" t="inlineStr">
+      <c r="M38" s="24" t="inlineStr">
         <is>
           <t>CBAM zboží (ocelové matice, kap. 73). Příjemce v registru: Y137 (do 50 t ročně). Díl 029-2513-AL-CZ – přípona 'AL' může znamenat HLINÍK → pak 7616 10 00 (také CBAM). Antidumping na spojovací prvky z CN (nař. 2022/191) se týká šroubů/vrutů, NE matic 7318 16 → AD neočekáváno (ověřit). Melt and pour: hutní atest CHYBÍ.</t>
         </is>
@@ -1989,9 +1992,9 @@
           <t>7318169290</t>
         </is>
       </c>
-      <c r="D39" s="12" t="inlineStr">
-        <is>
-          <t>Nut  ← faktura: "Nut"</t>
+      <c r="D39" s="18" t="inlineStr">
+        <is>
+          <t>Matice ⚠ (CZ popis není v ref. souboru klienta)  ← faktura: "Nut"</t>
         </is>
       </c>
       <c r="E39" s="14" t="n">
@@ -2038,8 +2041,8 @@
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>• Membrána s vlnkou  ← faktura: "Cone" – 58 680 ks | NW 964,310 kg | GW 1 324,030 kg | 22 202,70 EUR
-• Kopulka= krycí vložka  ← faktura: "Dust cap" – 52 000 ks | NW 12,600 kg | GW 17,100 kg | 8 034,00 EUR</t>
+          <t>• Membrána s vlnkou
+• Kopulka= krycí vložka</t>
         </is>
       </c>
       <c r="E40" s="8" t="n">
@@ -2312,35 +2315,35 @@
       <c r="M45" s="12" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="24" t="inlineStr">
+      <c r="A46" s="25" t="inlineStr">
         <is>
           <t>CELKEM</t>
         </is>
       </c>
-      <c r="B46" s="25" t="n"/>
-      <c r="C46" s="25" t="n"/>
-      <c r="D46" s="25" t="n"/>
-      <c r="E46" s="26">
+      <c r="B46" s="26" t="n"/>
+      <c r="C46" s="26" t="n"/>
+      <c r="D46" s="26" t="n"/>
+      <c r="E46" s="27">
         <f>E14+E22+E26+E35+E38+E40</f>
         <v/>
       </c>
-      <c r="F46" s="27">
+      <c r="F46" s="28">
         <f>F14+F22+F26+F35+F38+F40</f>
         <v/>
       </c>
-      <c r="G46" s="27">
+      <c r="G46" s="28">
         <f>G14+G22+G26+G35+G38+G40</f>
         <v/>
       </c>
-      <c r="H46" s="28">
+      <c r="H46" s="29">
         <f>H14+H22+H26+H35+H38+H40</f>
         <v/>
       </c>
-      <c r="I46" s="25" t="n"/>
-      <c r="J46" s="25" t="n"/>
-      <c r="K46" s="25" t="n"/>
-      <c r="L46" s="25" t="n"/>
-      <c r="M46" s="25" t="n"/>
+      <c r="I46" s="26" t="n"/>
+      <c r="J46" s="26" t="n"/>
+      <c r="K46" s="26" t="n"/>
+      <c r="L46" s="26" t="n"/>
+      <c r="M46" s="26" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -2410,7 +2413,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Nutno ověřit (popis/zařazení, Incoterm místo, hutní atest)</t>
+          <t>Nutno ověřit (popis/zařazení, Incoterm místo, hutní atest). ⚠ = český popis není v ref. souboru klienta – doplněn námi</t>
         </is>
       </c>
     </row>
@@ -2459,1331 +2462,1331 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="29" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t>Odesílatel</t>
         </is>
       </c>
-      <c r="B1" s="29" t="inlineStr">
+      <c r="B1" s="30" t="inlineStr">
         <is>
           <t>Faktura</t>
         </is>
       </c>
-      <c r="C1" s="29" t="inlineStr">
+      <c r="C1" s="30" t="inlineStr">
         <is>
           <t>Part number</t>
         </is>
       </c>
-      <c r="D1" s="29" t="inlineStr">
+      <c r="D1" s="30" t="inlineStr">
         <is>
           <t>Popis (faktura, EN)</t>
         </is>
       </c>
-      <c r="E1" s="29" t="inlineStr">
+      <c r="E1" s="30" t="inlineStr">
         <is>
           <t>HS kód</t>
         </is>
       </c>
-      <c r="F1" s="29" t="inlineStr">
+      <c r="F1" s="30" t="inlineStr">
         <is>
           <t>Popis CZ (klient)</t>
         </is>
       </c>
-      <c r="G1" s="29" t="inlineStr">
+      <c r="G1" s="30" t="inlineStr">
         <is>
           <t>Množství (ks)</t>
         </is>
       </c>
-      <c r="H1" s="29" t="inlineStr">
+      <c r="H1" s="30" t="inlineStr">
         <is>
           <t>Čistá hm. (kg)</t>
         </is>
       </c>
-      <c r="I1" s="29" t="inlineStr">
+      <c r="I1" s="30" t="inlineStr">
         <is>
           <t>Hrubá hm. (kg)</t>
         </is>
       </c>
-      <c r="J1" s="29" t="inlineStr">
+      <c r="J1" s="30" t="inlineStr">
         <is>
           <t>Částka EUR</t>
         </is>
       </c>
-      <c r="K1" s="29" t="inlineStr">
+      <c r="K1" s="30" t="inlineStr">
         <is>
           <t>Zdroj</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="30" t="inlineStr">
+      <c r="A2" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B2" s="30" t="inlineStr">
+      <c r="B2" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C2" s="30" t="inlineStr">
+      <c r="C2" s="31" t="inlineStr">
         <is>
           <t>IM-SW6515-VWCZ</t>
         </is>
       </c>
-      <c r="D2" s="30" t="inlineStr">
+      <c r="D2" s="31" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E2" s="31" t="inlineStr">
+      <c r="E2" s="32" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F2" s="30" t="inlineStr">
+      <c r="F2" s="31" t="inlineStr">
         <is>
           <t>Subwoofer</t>
         </is>
       </c>
-      <c r="G2" s="30" t="n">
+      <c r="G2" s="31" t="n">
         <v>540</v>
       </c>
-      <c r="H2" s="30" t="n">
+      <c r="H2" s="31" t="n">
         <v>313.2</v>
       </c>
-      <c r="I2" s="30" t="n">
+      <c r="I2" s="31" t="n">
         <v>350</v>
       </c>
-      <c r="J2" s="30" t="n">
+      <c r="J2" s="31" t="n">
         <v>2381.4</v>
       </c>
-      <c r="K2" s="30" t="inlineStr">
+      <c r="K2" s="31" t="inlineStr">
         <is>
           <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="30" t="inlineStr">
+      <c r="A3" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B3" s="30" t="inlineStr">
+      <c r="B3" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C3" s="30" t="inlineStr">
+      <c r="C3" s="31" t="inlineStr">
         <is>
           <t>IM-40138L-BMWCZ</t>
         </is>
       </c>
-      <c r="D3" s="30" t="inlineStr">
+      <c r="D3" s="31" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E3" s="31" t="inlineStr">
+      <c r="E3" s="32" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F3" s="30" t="inlineStr">
-        <is>
-          <t>Hotové reproduktory - ostatní</t>
-        </is>
-      </c>
-      <c r="G3" s="30" t="n">
+      <c r="F3" s="31" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory</t>
+        </is>
+      </c>
+      <c r="G3" s="31" t="n">
         <v>540</v>
       </c>
-      <c r="H3" s="30" t="n">
+      <c r="H3" s="31" t="n">
         <v>253.8</v>
       </c>
-      <c r="I3" s="30" t="n">
+      <c r="I3" s="31" t="n">
         <v>270</v>
       </c>
-      <c r="J3" s="30" t="n">
+      <c r="J3" s="31" t="n">
         <v>4594.21</v>
       </c>
-      <c r="K3" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+      <c r="K3" s="31" t="inlineStr">
+        <is>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="30" t="inlineStr">
+      <c r="A4" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B4" s="30" t="inlineStr">
+      <c r="B4" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C4" s="30" t="inlineStr">
+      <c r="C4" s="31" t="inlineStr">
         <is>
           <t>IM-65220G-BYCZ</t>
         </is>
       </c>
-      <c r="D4" s="30" t="inlineStr">
+      <c r="D4" s="31" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E4" s="31" t="inlineStr">
+      <c r="E4" s="32" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F4" s="30" t="inlineStr">
-        <is>
-          <t>Hotové reproduktory - ostatní</t>
-        </is>
-      </c>
-      <c r="G4" s="30" t="n">
+      <c r="F4" s="31" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory</t>
+        </is>
+      </c>
+      <c r="G4" s="31" t="n">
         <v>360</v>
       </c>
-      <c r="H4" s="30" t="n">
+      <c r="H4" s="31" t="n">
         <v>270</v>
       </c>
-      <c r="I4" s="30" t="n">
+      <c r="I4" s="31" t="n">
         <v>308</v>
       </c>
-      <c r="J4" s="30" t="n">
+      <c r="J4" s="31" t="n">
         <v>3623.72</v>
       </c>
-      <c r="K4" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+      <c r="K4" s="31" t="inlineStr">
+        <is>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B5" s="30" t="inlineStr">
+      <c r="B5" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C5" s="30" t="inlineStr">
+      <c r="C5" s="31" t="inlineStr">
         <is>
           <t>IM-SW6550-SKCZ</t>
         </is>
       </c>
-      <c r="D5" s="30" t="inlineStr">
+      <c r="D5" s="31" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E5" s="31" t="inlineStr">
+      <c r="E5" s="32" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F5" s="30" t="inlineStr">
+      <c r="F5" s="31" t="inlineStr">
         <is>
           <t>Subwoofer</t>
         </is>
       </c>
-      <c r="G5" s="30" t="n">
+      <c r="G5" s="31" t="n">
         <v>540</v>
       </c>
-      <c r="H5" s="30" t="n">
+      <c r="H5" s="31" t="n">
         <v>664.2</v>
       </c>
-      <c r="I5" s="30" t="n">
+      <c r="I5" s="31" t="n">
         <v>705.8200000000001</v>
       </c>
-      <c r="J5" s="30" t="n">
+      <c r="J5" s="31" t="n">
         <v>3607.2</v>
       </c>
-      <c r="K5" s="30" t="inlineStr">
+      <c r="K5" s="31" t="inlineStr">
         <is>
           <t>List1 ř.11 'Subwoofer' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="A6" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B6" s="30" t="inlineStr">
+      <c r="B6" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C6" s="30" t="inlineStr">
+      <c r="C6" s="31" t="inlineStr">
         <is>
           <t>212-8061-1-CZ</t>
         </is>
       </c>
-      <c r="D6" s="30" t="inlineStr">
+      <c r="D6" s="31" t="inlineStr">
         <is>
           <t>Speaker component</t>
         </is>
       </c>
-      <c r="E6" s="31" t="inlineStr">
+      <c r="E6" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F6" s="30" t="inlineStr">
-        <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
-        </is>
-      </c>
-      <c r="G6" s="30" t="n">
+      <c r="F6" s="31" t="inlineStr">
+        <is>
+          <t>magnetický obvod</t>
+        </is>
+      </c>
+      <c r="G6" s="31" t="n">
         <v>4608</v>
       </c>
-      <c r="H6" s="30" t="n">
+      <c r="H6" s="31" t="n">
         <v>2211.84</v>
       </c>
-      <c r="I6" s="30" t="n">
+      <c r="I6" s="31" t="n">
         <v>2312</v>
       </c>
-      <c r="J6" s="30" t="n">
+      <c r="J6" s="31" t="n">
         <v>3170.3</v>
       </c>
-      <c r="K6" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.2 (obecná položka)</t>
+      <c r="K6" s="31" t="inlineStr">
+        <is>
+          <t>List2 ř.37 'magnetický obvod'; řada 212-* = magnetový obvod (List1 ř.3: 212-65163-CZ)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B7" s="30" t="inlineStr">
+      <c r="B7" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C7" s="30" t="inlineStr">
+      <c r="C7" s="31" t="inlineStr">
         <is>
           <t>IM-65386-BYCZ</t>
         </is>
       </c>
-      <c r="D7" s="30" t="inlineStr">
+      <c r="D7" s="31" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E7" s="31" t="inlineStr">
+      <c r="E7" s="32" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F7" s="30" t="inlineStr">
-        <is>
-          <t>Hotové reproduktory - ostatní</t>
-        </is>
-      </c>
-      <c r="G7" s="30" t="n">
+      <c r="F7" s="31" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory</t>
+        </is>
+      </c>
+      <c r="G7" s="31" t="n">
         <v>240</v>
       </c>
-      <c r="H7" s="30" t="n">
+      <c r="H7" s="31" t="n">
         <v>175.2</v>
       </c>
-      <c r="I7" s="30" t="n">
+      <c r="I7" s="31" t="n">
         <v>195</v>
       </c>
-      <c r="J7" s="30" t="n">
+      <c r="J7" s="31" t="n">
         <v>2058.46</v>
       </c>
-      <c r="K7" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+      <c r="K7" s="31" t="inlineStr">
+        <is>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="A8" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B8" s="30" t="inlineStr">
+      <c r="B8" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C8" s="30" t="inlineStr">
+      <c r="C8" s="31" t="inlineStr">
         <is>
           <t>IM-65387-BYCZ</t>
         </is>
       </c>
-      <c r="D8" s="30" t="inlineStr">
+      <c r="D8" s="31" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E8" s="31" t="inlineStr">
+      <c r="E8" s="32" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F8" s="30" t="inlineStr">
-        <is>
-          <t>Hotové reproduktory - ostatní</t>
-        </is>
-      </c>
-      <c r="G8" s="30" t="n">
+      <c r="F8" s="31" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory</t>
+        </is>
+      </c>
+      <c r="G8" s="31" t="n">
         <v>180</v>
       </c>
-      <c r="H8" s="30" t="n">
+      <c r="H8" s="31" t="n">
         <v>133.2</v>
       </c>
-      <c r="I8" s="30" t="n">
+      <c r="I8" s="31" t="n">
         <v>152</v>
       </c>
-      <c r="J8" s="30" t="n">
+      <c r="J8" s="31" t="n">
         <v>1802.86</v>
       </c>
-      <c r="K8" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+      <c r="K8" s="31" t="inlineStr">
+        <is>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B9" s="30" t="inlineStr">
+      <c r="B9" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C9" s="30" t="inlineStr">
+      <c r="C9" s="31" t="inlineStr">
         <is>
           <t>IM-40137L-BMWCZ</t>
         </is>
       </c>
-      <c r="D9" s="30" t="inlineStr">
+      <c r="D9" s="31" t="inlineStr">
         <is>
           <t>Car Speaker</t>
         </is>
       </c>
-      <c r="E9" s="31" t="inlineStr">
+      <c r="E9" s="32" t="inlineStr">
         <is>
           <t>8518290090</t>
         </is>
       </c>
-      <c r="F9" s="30" t="inlineStr">
-        <is>
-          <t>Hotové reproduktory - ostatní</t>
-        </is>
-      </c>
-      <c r="G9" s="30" t="n">
+      <c r="F9" s="31" t="inlineStr">
+        <is>
+          <t>Hotové reproduktory</t>
+        </is>
+      </c>
+      <c r="G9" s="31" t="n">
         <v>540</v>
       </c>
-      <c r="H9" s="30" t="n">
+      <c r="H9" s="31" t="n">
         <v>253.8</v>
       </c>
-      <c r="I9" s="30" t="n">
+      <c r="I9" s="31" t="n">
         <v>270</v>
       </c>
-      <c r="J9" s="30" t="n">
+      <c r="J9" s="31" t="n">
         <v>4199.09</v>
       </c>
-      <c r="K9" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.10 + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
+      <c r="K9" s="31" t="inlineStr">
+        <is>
+          <t>List1 ř.9–10 'Hotové reproduktory' + List2 ř.197 ('tohle řadíme pod 8518290090')</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="A10" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B10" s="30" t="inlineStr">
+      <c r="B10" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C10" s="30" t="inlineStr">
+      <c r="C10" s="31" t="inlineStr">
         <is>
           <t>212-65424-CZ</t>
         </is>
       </c>
-      <c r="D10" s="30" t="inlineStr">
+      <c r="D10" s="31" t="inlineStr">
         <is>
           <t>Speaker component</t>
         </is>
       </c>
-      <c r="E10" s="31" t="inlineStr">
+      <c r="E10" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F10" s="30" t="inlineStr">
-        <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
-        </is>
-      </c>
-      <c r="G10" s="30" t="n">
+      <c r="F10" s="31" t="inlineStr">
+        <is>
+          <t>magnetický obvod</t>
+        </is>
+      </c>
+      <c r="G10" s="31" t="n">
         <v>7680</v>
       </c>
-      <c r="H10" s="30" t="n">
+      <c r="H10" s="31" t="n">
         <v>1766.4</v>
       </c>
-      <c r="I10" s="30" t="n">
+      <c r="I10" s="31" t="n">
         <v>1797.6</v>
       </c>
-      <c r="J10" s="30" t="n">
+      <c r="J10" s="31" t="n">
         <v>1831.68</v>
       </c>
-      <c r="K10" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.2 (obecná položka)</t>
+      <c r="K10" s="31" t="inlineStr">
+        <is>
+          <t>List2 ř.37 'magnetický obvod'; řada 212-* = magnetový obvod (List1 ř.3: 212-65163-CZ)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox Electronics Co., Ltd</t>
         </is>
       </c>
-      <c r="B11" s="30" t="inlineStr">
+      <c r="B11" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-1</t>
         </is>
       </c>
-      <c r="C11" s="30" t="inlineStr">
+      <c r="C11" s="31" t="inlineStr">
         <is>
           <t>212-65581-CZ</t>
         </is>
       </c>
-      <c r="D11" s="30" t="inlineStr">
+      <c r="D11" s="31" t="inlineStr">
         <is>
           <t>Speaker component</t>
         </is>
       </c>
-      <c r="E11" s="31" t="inlineStr">
+      <c r="E11" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F11" s="30" t="inlineStr">
-        <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
-        </is>
-      </c>
-      <c r="G11" s="30" t="n">
+      <c r="F11" s="31" t="inlineStr">
+        <is>
+          <t>magnetický obvod</t>
+        </is>
+      </c>
+      <c r="G11" s="31" t="n">
         <v>1053</v>
       </c>
-      <c r="H11" s="30" t="n">
+      <c r="H11" s="31" t="n">
         <v>452.79</v>
       </c>
-      <c r="I11" s="30" t="n">
+      <c r="I11" s="31" t="n">
         <v>489.32</v>
       </c>
-      <c r="J11" s="30" t="n">
+      <c r="J11" s="31" t="n">
         <v>694.98</v>
       </c>
-      <c r="K11" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.2 (obecná položka)</t>
+      <c r="K11" s="31" t="inlineStr">
+        <is>
+          <t>List2 ř.37 'magnetický obvod'; řada 212-* = magnetový obvod (List1 ř.3: 212-65163-CZ)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="A12" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B12" s="30" t="inlineStr">
+      <c r="B12" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C12" s="30" t="inlineStr">
+      <c r="C12" s="31" t="inlineStr">
         <is>
           <t>040-65E4-C-CZ</t>
         </is>
       </c>
-      <c r="D12" s="30" t="inlineStr">
+      <c r="D12" s="31" t="inlineStr">
         <is>
           <t>Front plate</t>
         </is>
       </c>
-      <c r="E12" s="31" t="inlineStr">
+      <c r="E12" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F12" s="30" t="inlineStr">
-        <is>
-          <t>ocelová deska</t>
-        </is>
-      </c>
-      <c r="G12" s="30" t="n">
+      <c r="F12" s="31" t="inlineStr">
+        <is>
+          <t>ocelová deska (přední deska)</t>
+        </is>
+      </c>
+      <c r="G12" s="31" t="n">
         <v>3000</v>
       </c>
-      <c r="H12" s="30" t="n">
+      <c r="H12" s="31" t="n">
         <v>222</v>
       </c>
-      <c r="I12" s="30" t="n">
+      <c r="I12" s="31" t="n">
         <v>225.43</v>
       </c>
-      <c r="J12" s="30" t="n">
+      <c r="J12" s="31" t="n">
         <v>309.9</v>
       </c>
-      <c r="K12" s="30" t="inlineStr">
+      <c r="K12" s="31" t="inlineStr">
         <is>
           <t>List2 ř.14 (+ dřívější JSD 85189000 00)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="A13" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B13" s="30" t="inlineStr">
+      <c r="B13" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C13" s="30" t="inlineStr">
+      <c r="C13" s="31" t="inlineStr">
         <is>
           <t>210-50D3-17.5TCR-CZ</t>
         </is>
       </c>
-      <c r="D13" s="30" t="inlineStr">
+      <c r="D13" s="31" t="inlineStr">
         <is>
           <t>T-yoke</t>
         </is>
       </c>
-      <c r="E13" s="31" t="inlineStr">
+      <c r="E13" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F13" s="30" t="inlineStr">
+      <c r="F13" s="31" t="inlineStr">
         <is>
           <t>jádro magnetického obvodu</t>
         </is>
       </c>
-      <c r="G13" s="30" t="n">
+      <c r="G13" s="31" t="n">
         <v>17160</v>
       </c>
-      <c r="H13" s="30" t="n">
+      <c r="H13" s="31" t="n">
         <v>1115.4</v>
       </c>
-      <c r="I13" s="30" t="n">
+      <c r="I13" s="31" t="n">
         <v>1155.4</v>
       </c>
-      <c r="J13" s="30" t="n">
+      <c r="J13" s="31" t="n">
         <v>1395.11</v>
       </c>
-      <c r="K13" s="30" t="inlineStr">
+      <c r="K13" s="31" t="inlineStr">
         <is>
           <t>List2 ř.23</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B14" s="30" t="inlineStr">
+      <c r="B14" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C14" s="30" t="inlineStr">
+      <c r="C14" s="31" t="inlineStr">
         <is>
           <t>021-88E00-9-2-CZ</t>
         </is>
       </c>
-      <c r="D14" s="30" t="inlineStr">
+      <c r="D14" s="31" t="inlineStr">
         <is>
           <t>Spider</t>
         </is>
       </c>
-      <c r="E14" s="31" t="inlineStr">
+      <c r="E14" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F14" s="30" t="inlineStr">
+      <c r="F14" s="31" t="inlineStr">
         <is>
           <t>Středící membrána</t>
         </is>
       </c>
-      <c r="G14" s="30" t="n">
+      <c r="G14" s="31" t="n">
         <v>3000</v>
       </c>
-      <c r="H14" s="30" t="n">
+      <c r="H14" s="31" t="n">
         <v>4.5</v>
       </c>
-      <c r="I14" s="30" t="n">
+      <c r="I14" s="31" t="n">
         <v>9.5</v>
       </c>
-      <c r="J14" s="30" t="n">
+      <c r="J14" s="31" t="n">
         <v>282.6</v>
       </c>
-      <c r="K14" s="30" t="inlineStr">
+      <c r="K14" s="31" t="inlineStr">
         <is>
           <t>List2 ř.7</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="30" t="inlineStr">
+      <c r="A15" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B15" s="30" t="inlineStr">
+      <c r="B15" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C15" s="30" t="inlineStr">
+      <c r="C15" s="31" t="inlineStr">
         <is>
           <t>142-530H10-10H-CZ</t>
         </is>
       </c>
-      <c r="D15" s="30" t="inlineStr">
+      <c r="D15" s="31" t="inlineStr">
         <is>
           <t>Gasket</t>
         </is>
       </c>
-      <c r="E15" s="31" t="inlineStr">
+      <c r="E15" s="32" t="inlineStr">
         <is>
           <t>3926909790</t>
         </is>
       </c>
-      <c r="F15" s="30" t="inlineStr">
+      <c r="F15" s="31" t="inlineStr">
         <is>
           <t>plastové těsnění</t>
         </is>
       </c>
-      <c r="G15" s="30" t="n">
+      <c r="G15" s="31" t="n">
         <v>3000</v>
       </c>
-      <c r="H15" s="30" t="n">
+      <c r="H15" s="31" t="n">
         <v>22.5</v>
       </c>
-      <c r="I15" s="30" t="n">
+      <c r="I15" s="31" t="n">
         <v>27.5</v>
       </c>
-      <c r="J15" s="30" t="n">
+      <c r="J15" s="31" t="n">
         <v>126</v>
       </c>
-      <c r="K15" s="30" t="inlineStr">
+      <c r="K15" s="31" t="inlineStr">
         <is>
           <t>List2 ř.50 (39269097); díly 142-*, ne 143-* (gumové)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="30" t="inlineStr">
+      <c r="A16" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B16" s="30" t="inlineStr">
+      <c r="B16" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C16" s="30" t="inlineStr">
+      <c r="C16" s="31" t="inlineStr">
         <is>
           <t>142-65580-3A-CZ</t>
         </is>
       </c>
-      <c r="D16" s="30" t="inlineStr">
+      <c r="D16" s="31" t="inlineStr">
         <is>
           <t>Gasket</t>
         </is>
       </c>
-      <c r="E16" s="31" t="inlineStr">
+      <c r="E16" s="32" t="inlineStr">
         <is>
           <t>3926909790</t>
         </is>
       </c>
-      <c r="F16" s="30" t="inlineStr">
+      <c r="F16" s="31" t="inlineStr">
         <is>
           <t>plastové těsnění</t>
         </is>
       </c>
-      <c r="G16" s="30" t="n">
+      <c r="G16" s="31" t="n">
         <v>3000</v>
       </c>
-      <c r="H16" s="30" t="n">
+      <c r="H16" s="31" t="n">
         <v>22.5</v>
       </c>
-      <c r="I16" s="30" t="n">
+      <c r="I16" s="31" t="n">
         <v>27.5</v>
       </c>
-      <c r="J16" s="30" t="n">
+      <c r="J16" s="31" t="n">
         <v>144</v>
       </c>
-      <c r="K16" s="30" t="inlineStr">
+      <c r="K16" s="31" t="inlineStr">
         <is>
           <t>List2 ř.50 (39269097); díly 142-*, ne 143-* (gumové)</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="A17" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B17" s="30" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C17" s="30" t="inlineStr">
+      <c r="C17" s="31" t="inlineStr">
         <is>
           <t>181-40133-1SN-CZ</t>
         </is>
       </c>
-      <c r="D17" s="30" t="inlineStr">
+      <c r="D17" s="31" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="E17" s="31" t="inlineStr">
+      <c r="E17" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F17" s="30" t="inlineStr">
+      <c r="F17" s="31" t="inlineStr">
         <is>
           <t>Terminál</t>
         </is>
       </c>
-      <c r="G17" s="30" t="n">
+      <c r="G17" s="31" t="n">
         <v>150000</v>
       </c>
-      <c r="H17" s="30" t="n">
+      <c r="H17" s="31" t="n">
         <v>75</v>
       </c>
-      <c r="I17" s="30" t="n">
+      <c r="I17" s="31" t="n">
         <v>80</v>
       </c>
-      <c r="J17" s="30" t="n">
+      <c r="J17" s="31" t="n">
         <v>1905</v>
       </c>
-      <c r="K17" s="30" t="inlineStr">
+      <c r="K17" s="31" t="inlineStr">
         <is>
           <t>List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="A18" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B18" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C18" s="30" t="inlineStr">
+      <c r="C18" s="31" t="inlineStr">
         <is>
           <t>181-40133-2SN-CZ</t>
         </is>
       </c>
-      <c r="D18" s="30" t="inlineStr">
+      <c r="D18" s="31" t="inlineStr">
         <is>
           <t>Terminal</t>
         </is>
       </c>
-      <c r="E18" s="31" t="inlineStr">
+      <c r="E18" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F18" s="30" t="inlineStr">
+      <c r="F18" s="31" t="inlineStr">
         <is>
           <t>Terminál</t>
         </is>
       </c>
-      <c r="G18" s="30" t="n">
+      <c r="G18" s="31" t="n">
         <v>150000</v>
       </c>
-      <c r="H18" s="30" t="n">
+      <c r="H18" s="31" t="n">
         <v>75</v>
       </c>
-      <c r="I18" s="30" t="n">
+      <c r="I18" s="31" t="n">
         <v>80</v>
       </c>
-      <c r="J18" s="30" t="n">
+      <c r="J18" s="31" t="n">
         <v>1905</v>
       </c>
-      <c r="K18" s="30" t="inlineStr">
+      <c r="K18" s="31" t="inlineStr">
         <is>
           <t>List2 ř.51 + ř.205 (díl 181-40133-1SN-CZ)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="A19" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B19" s="30" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C19" s="30" t="inlineStr">
+      <c r="C19" s="31" t="inlineStr">
         <is>
           <t>029-2513-AL-CZ</t>
         </is>
       </c>
-      <c r="D19" s="30" t="inlineStr">
+      <c r="D19" s="31" t="inlineStr">
         <is>
           <t>Nut</t>
         </is>
       </c>
-      <c r="E19" s="31" t="inlineStr">
+      <c r="E19" s="32" t="inlineStr">
         <is>
           <t>7318169290</t>
         </is>
       </c>
-      <c r="F19" s="30" t="inlineStr">
-        <is>
-          <t>Nut</t>
-        </is>
-      </c>
-      <c r="G19" s="30" t="n">
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>Matice</t>
+        </is>
+      </c>
+      <c r="G19" s="31" t="n">
         <v>100000</v>
       </c>
-      <c r="H19" s="30" t="n">
+      <c r="H19" s="31" t="n">
         <v>166.5</v>
       </c>
-      <c r="I19" s="30" t="n">
+      <c r="I19" s="31" t="n">
         <v>172.5</v>
       </c>
-      <c r="J19" s="30" t="n">
+      <c r="J19" s="31" t="n">
         <v>7000</v>
       </c>
-      <c r="K19" s="30" t="inlineStr">
+      <c r="K19" s="31" t="inlineStr">
         <is>
           <t>List2 ř.202 ('tohle řadíme pod 7318169290') – bez CZ popisu</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="30" t="inlineStr">
+      <c r="A20" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B20" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C20" s="30" t="inlineStr">
+      <c r="C20" s="31" t="inlineStr">
         <is>
           <t>140-35D14-44XP1-CZ</t>
         </is>
       </c>
-      <c r="D20" s="30" t="inlineStr">
+      <c r="D20" s="31" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E20" s="31" t="inlineStr">
+      <c r="E20" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F20" s="30" t="inlineStr">
+      <c r="F20" s="31" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G20" s="30" t="n">
+      <c r="G20" s="31" t="n">
         <v>34000</v>
       </c>
-      <c r="H20" s="30" t="n">
+      <c r="H20" s="31" t="n">
         <v>68</v>
       </c>
-      <c r="I20" s="30" t="n">
+      <c r="I20" s="31" t="n">
         <v>130</v>
       </c>
-      <c r="J20" s="30" t="n">
+      <c r="J20" s="31" t="n">
         <v>12437.2</v>
       </c>
-      <c r="K20" s="30" t="inlineStr">
+      <c r="K20" s="31" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="30" t="inlineStr">
+      <c r="A21" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B21" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C21" s="30" t="inlineStr">
+      <c r="C21" s="31" t="inlineStr">
         <is>
           <t>015-S753215-Y30-KS-CZ</t>
         </is>
       </c>
-      <c r="D21" s="30" t="inlineStr">
+      <c r="D21" s="31" t="inlineStr">
         <is>
           <t>Speaker components</t>
         </is>
       </c>
-      <c r="E21" s="31" t="inlineStr">
+      <c r="E21" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F21" s="30" t="inlineStr">
-        <is>
-          <t>Komponenty pro výrobu autoreproduktorů - Ostatní - všechny položky, kromě vyjmenovaných níže</t>
-        </is>
-      </c>
-      <c r="G21" s="30" t="n">
+      <c r="F21" s="31" t="inlineStr">
+        <is>
+          <t>Feritový magnet</t>
+        </is>
+      </c>
+      <c r="G21" s="31" t="n">
         <v>21600</v>
       </c>
-      <c r="H21" s="30" t="n">
+      <c r="H21" s="31" t="n">
         <v>5616</v>
       </c>
-      <c r="I21" s="30" t="n">
+      <c r="I21" s="31" t="n">
         <v>5736</v>
       </c>
-      <c r="J21" s="30" t="n">
+      <c r="J21" s="31" t="n">
         <v>5978.88</v>
       </c>
-      <c r="K21" s="30" t="inlineStr">
-        <is>
-          <t>List1 ř.2 (obecná položka)</t>
+      <c r="K21" s="31" t="inlineStr">
+        <is>
+          <t>List2 ř.29 'MAGNET' 8518900000 – CZ popis v ref. souboru NENÍ (S753215 = kroužek 75×32×15 mm, Y30 = ferit)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="30" t="inlineStr">
+      <c r="A22" s="31" t="inlineStr">
         <is>
           <t>Suzhou Sonavox International Trading Co., Ltd</t>
         </is>
       </c>
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B22" s="31" t="inlineStr">
         <is>
           <t>CZ20260904</t>
         </is>
       </c>
-      <c r="C22" s="30" t="inlineStr">
+      <c r="C22" s="31" t="inlineStr">
         <is>
           <t>210-66E2-24.5TCR-1-CZ</t>
         </is>
       </c>
-      <c r="D22" s="30" t="inlineStr">
+      <c r="D22" s="31" t="inlineStr">
         <is>
           <t>T-yoke</t>
         </is>
       </c>
-      <c r="E22" s="31" t="inlineStr">
+      <c r="E22" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F22" s="30" t="inlineStr">
+      <c r="F22" s="31" t="inlineStr">
         <is>
           <t>jádro magnetického obvodu</t>
         </is>
       </c>
-      <c r="G22" s="30" t="n">
+      <c r="G22" s="31" t="n">
         <v>42840</v>
       </c>
-      <c r="H22" s="30" t="n">
+      <c r="H22" s="31" t="n">
         <v>6897.24</v>
       </c>
-      <c r="I22" s="30" t="n">
+      <c r="I22" s="31" t="n">
         <v>7037.24</v>
       </c>
-      <c r="J22" s="30" t="n">
+      <c r="J22" s="31" t="n">
         <v>8186.72</v>
       </c>
-      <c r="K22" s="30" t="inlineStr">
+      <c r="K22" s="31" t="inlineStr">
         <is>
           <t>List2 ř.23</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B23" s="30" t="inlineStr">
+      <c r="B23" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C23" s="30" t="inlineStr">
+      <c r="C23" s="31" t="inlineStr">
         <is>
           <t>140-65D24-179X-CZ</t>
         </is>
       </c>
-      <c r="D23" s="30" t="inlineStr">
+      <c r="D23" s="31" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E23" s="31" t="inlineStr">
+      <c r="E23" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F23" s="30" t="inlineStr">
+      <c r="F23" s="31" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G23" s="30" t="n">
+      <c r="G23" s="31" t="n">
         <v>17280</v>
       </c>
-      <c r="H23" s="30" t="n">
+      <c r="H23" s="31" t="n">
         <v>240</v>
       </c>
-      <c r="I23" s="30" t="n">
+      <c r="I23" s="31" t="n">
         <v>373.33</v>
       </c>
-      <c r="J23" s="30" t="n">
+      <c r="J23" s="31" t="n">
         <v>4397.76</v>
       </c>
-      <c r="K23" s="30" t="inlineStr">
+      <c r="K23" s="31" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="30" t="inlineStr">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B24" s="30" t="inlineStr">
+      <c r="B24" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C24" s="30" t="inlineStr">
+      <c r="C24" s="31" t="inlineStr">
         <is>
           <t>140-80I27-42X-CZ</t>
         </is>
       </c>
-      <c r="D24" s="30" t="inlineStr">
+      <c r="D24" s="31" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E24" s="31" t="inlineStr">
+      <c r="E24" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F24" s="30" t="inlineStr">
+      <c r="F24" s="31" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G24" s="30" t="n">
+      <c r="G24" s="31" t="n">
         <v>24000</v>
       </c>
-      <c r="H24" s="30" t="n">
+      <c r="H24" s="31" t="n">
         <v>612</v>
       </c>
-      <c r="I24" s="30" t="n">
+      <c r="I24" s="31" t="n">
         <v>810</v>
       </c>
-      <c r="J24" s="30" t="n">
+      <c r="J24" s="31" t="n">
         <v>12026.4</v>
       </c>
-      <c r="K24" s="30" t="inlineStr">
+      <c r="K24" s="31" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="30" t="inlineStr">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B25" s="30" t="inlineStr">
+      <c r="B25" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C25" s="30" t="inlineStr">
+      <c r="C25" s="31" t="inlineStr">
         <is>
           <t>160-B29-H-CZ</t>
         </is>
       </c>
-      <c r="D25" s="30" t="inlineStr">
+      <c r="D25" s="31" t="inlineStr">
         <is>
           <t>Dust cap</t>
         </is>
       </c>
-      <c r="E25" s="31" t="inlineStr">
+      <c r="E25" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F25" s="30" t="inlineStr">
+      <c r="F25" s="31" t="inlineStr">
         <is>
           <t>Kopulka= krycí vložka</t>
         </is>
       </c>
-      <c r="G25" s="30" t="n">
+      <c r="G25" s="31" t="n">
         <v>52000</v>
       </c>
-      <c r="H25" s="30" t="n">
+      <c r="H25" s="31" t="n">
         <v>12.6</v>
       </c>
-      <c r="I25" s="30" t="n">
+      <c r="I25" s="31" t="n">
         <v>17.1</v>
       </c>
-      <c r="J25" s="30" t="n">
+      <c r="J25" s="31" t="n">
         <v>8034</v>
       </c>
-      <c r="K25" s="30" t="inlineStr">
+      <c r="K25" s="31" t="inlineStr">
         <is>
           <t>List2 ř.9 (uvedeno 8518 9000 99)</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="30" t="inlineStr">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B26" s="30" t="inlineStr">
+      <c r="B26" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C26" s="30" t="inlineStr">
+      <c r="C26" s="31" t="inlineStr">
         <is>
           <t>140-65E22-203X-CZ</t>
         </is>
       </c>
-      <c r="D26" s="30" t="inlineStr">
+      <c r="D26" s="31" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E26" s="31" t="inlineStr">
+      <c r="E26" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F26" s="30" t="inlineStr">
+      <c r="F26" s="31" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G26" s="30" t="n">
+      <c r="G26" s="31" t="n">
         <v>3000</v>
       </c>
-      <c r="H26" s="30" t="n">
+      <c r="H26" s="31" t="n">
         <v>25.91</v>
       </c>
-      <c r="I26" s="30" t="n">
+      <c r="I26" s="31" t="n">
         <v>39.36</v>
       </c>
-      <c r="J26" s="30" t="n">
+      <c r="J26" s="31" t="n">
         <v>895.5</v>
       </c>
-      <c r="K26" s="30" t="inlineStr">
+      <c r="K26" s="31" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="30" t="inlineStr">
+      <c r="A27" s="31" t="inlineStr">
         <is>
           <t>Suzhou Yanlong Electronic Product Co., Ltd</t>
         </is>
       </c>
-      <c r="B27" s="30" t="inlineStr">
+      <c r="B27" s="31" t="inlineStr">
         <is>
           <t>CZ20260904-2</t>
         </is>
       </c>
-      <c r="C27" s="30" t="inlineStr">
+      <c r="C27" s="31" t="inlineStr">
         <is>
           <t>140-40E17-72XC-CZ</t>
         </is>
       </c>
-      <c r="D27" s="30" t="inlineStr">
+      <c r="D27" s="31" t="inlineStr">
         <is>
           <t>Cone</t>
         </is>
       </c>
-      <c r="E27" s="31" t="inlineStr">
+      <c r="E27" s="32" t="inlineStr">
         <is>
           <t>8518900000</t>
         </is>
       </c>
-      <c r="F27" s="30" t="inlineStr">
+      <c r="F27" s="31" t="inlineStr">
         <is>
           <t>Membrána s vlnkou</t>
         </is>
       </c>
-      <c r="G27" s="30" t="n">
+      <c r="G27" s="31" t="n">
         <v>14400</v>
       </c>
-      <c r="H27" s="30" t="n">
+      <c r="H27" s="31" t="n">
         <v>86.40000000000001</v>
       </c>
-      <c r="I27" s="30" t="n">
+      <c r="I27" s="31" t="n">
         <v>101.34</v>
       </c>
-      <c r="J27" s="30" t="n">
+      <c r="J27" s="31" t="n">
         <v>4883.04</v>
       </c>
-      <c r="K27" s="30" t="inlineStr">
+      <c r="K27" s="31" t="inlineStr">
         <is>
           <t>List2 ř.8 / List1 ř.4</t>
         </is>
@@ -3800,196 +3803,210 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="160" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="32" t="inlineStr">
+      <c r="A1" s="33" t="inlineStr">
         <is>
           <t>PREFERENČNÍ VĚTA (COO)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="33" t="inlineStr">
+      <c r="A2" s="34" t="inlineStr">
         <is>
           <t>Na žádné ze 3 faktur NENÍ preferenční věta. Země původu Čína → bez preferencí, platí standardní clo (8518 90 00 0 %, 8518 29 3 %*, 3926 90 97 6,5 %, 7318 16 3,7 %).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="32" t="inlineStr">
+      <c r="A3" s="33" t="inlineStr">
         <is>
           <t>REX ČÍSLO</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="33" t="inlineStr">
+      <c r="A4" s="34" t="inlineStr">
         <is>
           <t>REX číslo NENÍ uvedeno na žádné faktuře (CZ20260904, CZ20260904-1, CZ20260904-2).</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="32" t="inlineStr">
+      <c r="A5" s="33" t="inlineStr">
         <is>
           <t>CBAM – příjemce Sonavox Technology CZ s.r.o.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="33" t="inlineStr">
+      <c r="A6" s="34" t="inlineStr">
         <is>
           <t>CBAM HS kód: 7318169290 (matice, 166,5 kg NW, odesílatel Suzhou Sonavox International Trading).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="33" t="inlineStr">
+      <c r="A7" s="34" t="inlineStr">
         <is>
           <t>Registr reference/CBAM_receivers_CZ.xlsx: 'Sonavox Technology CZ s.r.o.' NALEZEN → Y KÓD = Y137 (do 50 t ročně). Povolení: –, podaná žádost: –, datum vydání: neuvedeno.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="34" t="inlineStr">
+      <c r="A8" s="35" t="inlineStr">
         <is>
           <t>⚠ NESOULAD EORI: registr uvádí EORI CZ62908227, ale ref. soubor klienta uvádí 'EORI=DIČ=CZ28632389'. CZ62908227 je na FCR uvedeno jako VAT zasílatele (Maurice Ward &amp; Co.) → pravděpodobně chyba v registru, ověřit a opravit.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="33" t="inlineStr">
+      <c r="A9" s="34" t="inlineStr">
         <is>
           <t>Není to firma mimo EU na sdíleném účtu CBAM-CZ-2025-QGM67089385721.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="A10" s="33" t="inlineStr">
         <is>
           <t>MELT AND POUR (země tavby a odlití)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="34" t="inlineStr">
+      <c r="A11" s="35" t="inlineStr">
         <is>
           <t>CHYBÍ: v dokladech není hutní atest (mill test certificate) ani země tavby a odlití. Týká se ocelových matic 7318169290 (029-2513-AL-CZ, 100 000 ks, 166,5 kg) → vyžádat hutní atest před proclením.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="33" t="inlineStr">
+      <c r="A12" s="34" t="inlineStr">
         <is>
           <t>Ocelové díly zařazené jako díly reproduktorů 8518 90 00 (Front plate 'ocelová deska' 222 kg, T-yoke 'jádro magnetického obvodu' 8 012,64 kg) – mimo kap. 72/73, ale ocelové; hutní atest také není k dispozici – doporučuji vyžádat.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="33" t="inlineStr">
+      <c r="A13" s="34" t="inlineStr">
         <is>
           <t>Pokud se potvrdí, že matice jsou hliníkové ('AL'), melt and pour (ocel) se na ně nevztahuje, ale CBAM ano (7616 10 00).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="32" t="inlineStr">
+      <c r="A14" s="33" t="inlineStr">
         <is>
           <t>ANTIDUMPING</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="33" t="inlineStr">
+      <c r="A15" s="34" t="inlineStr">
         <is>
           <t>Žádná položka podle aktuálního zařazení nepodléhá antidumpingu. Matice 7318 16 nejsou v rozsahu AD cla na spojovací prvky z CN (šrouby 7318 15 – 86,5 % dle ref. klienta – v zásilce nejsou). Ověřit při podání JSD.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="32" t="inlineStr">
+      <c r="A16" s="33" t="inlineStr">
         <is>
           <t>INCOTERM</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="34" t="inlineStr">
+      <c r="A17" s="35" t="inlineStr">
         <is>
           <t>Faktury: 'Terms of Payment: FOB' – BEZ pojmenovaného místa. FCR: místo převzetí Wuhan, Hubei; FREIGHT COLLECT. FOB je námořní doložka, zde železnice → doplnit místo (FOB Wuhan? / Suzhou?) od klienta.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="32" t="inlineStr">
+      <c r="A18" s="33" t="inlineStr">
         <is>
           <t>HODNOTA – 'Total'</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="33" t="inlineStr">
+      <c r="A19" s="34" t="inlineStr">
         <is>
           <t>CZ20260904-1 (Sonavox Electronics): Total Amount = 27 963,90 EUR ✓.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="34" t="inlineStr">
+      <c r="A20" s="35" t="inlineStr">
         <is>
           <t>CZ20260904 (Sonavox International Trading) a CZ20260904-2 (Yanlong): řádek 'Total Amount' je PRÁZDNÝ; 'Total :' je jen u množství. Použit Sub Total 39 670,41 a 30 236,70 EUR (Duty/Freight/Insurance prázdné, bez slevy) – potvrdit.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="32" t="inlineStr">
+      <c r="A21" s="33" t="inlineStr">
         <is>
           <t>CCT/VPV KN</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="33" t="inlineStr">
+      <c r="A22" s="34" t="inlineStr">
         <is>
           <t>Pravidlo CCT/VPV KN nebylo použito – všechny položky mají HS kód v referenčním souboru klienta 'Celní zařazení obvyklých položek Sonavox'. Faktury samy HS kódy neuvádějí; CIM uvádí pro vše 8518900000.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="32" t="inlineStr">
+      <c r="A23" s="33" t="inlineStr">
         <is>
           <t>ZAŘAZENÍ K OVĚŘENÍ</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="33" t="inlineStr">
+      <c r="A24" s="34" t="inlineStr">
         <is>
           <t>Gasket (142-*) – plast 3926909790 vs. pryž 4016 vs. pěna 3921; materiál nepotvrzen.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="33" t="inlineStr">
-        <is>
-          <t>Nut (029-2513-AL-CZ) – klient nemá český popis; 'AL' → možná hliník (7616 10 00).</t>
+      <c r="A25" s="34" t="inlineStr">
+        <is>
+          <t>Nut (029-2513-AL-CZ) – klient nemá český popis → doplněno 'Matice' (náš překlad); 'AL' → možná hliník (7616 10 00).</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="33" t="inlineStr">
-        <is>
-          <t>Speaker components 015-S753215-Y30-KS-CZ (5 616 kg) – 'Y30' = feritová třída → spíše magnet (8505 19 dle Pozn. 2a tř. XVI) než 8518 90 00 – případně konzultovat s customs.tariff@mauriceward.com.</t>
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>Speaker components 015-S753215-Y30-KS-CZ – klient nemá český popis → doplněno 'Feritový magnet' (náš popis dle rozměru 75×32×15 mm a třídy Y30).</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="33" t="inlineStr">
+      <c r="A27" s="34" t="inlineStr">
+        <is>
+          <t>Speaker component 212-* – faktura bez bližšího popisu → 'magnetický obvod' dle řady part number 212-* v ref. souboru klienta; potvrdit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="34" t="inlineStr">
+        <is>
+          <t>Feritový magnet 015-S753215-Y30-KS-CZ (5 616 kg) – jako magnet patří spíše pod 8505 19 (Pozn. 2a k tř. XVI) než pod 8518 90 00 – případně konzultovat s customs.tariff@mauriceward.com.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="34" t="inlineStr">
         <is>
           <t>Car speakers – 8518290090 (poslední poznámka klienta) vs. 8518 29 95 (List1). *Sazba 3 % dle List1 – ověřit v TARIC.</t>
         </is>

</xml_diff>